<commit_message>
change tables into 4 d.p.
</commit_message>
<xml_diff>
--- a/output/coefficients/standardized/standardized_ALL.xlsx
+++ b/output/coefficients/standardized/standardized_ALL.xlsx
@@ -464,15 +464,15 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.4783288253257217</v>
+        <v>0.4783</v>
       </c>
       <c r="C2" t="n">
-        <v>0.01030794414712172</v>
+        <v>0.0103</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>46.40390154415856</v>
+        <v>46.4039</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -485,19 +485,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1114987810552704</v>
+        <v>0.1115</v>
       </c>
       <c r="C3" t="n">
-        <v>0.004931284352144412</v>
+        <v>0.0049</v>
       </c>
       <c r="D3" t="n">
-        <v>0.241216519582306</v>
+        <v>0.2412</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01066834307278497</v>
+        <v>0.0107</v>
       </c>
       <c r="F3" t="n">
-        <v>22.61049517592393</v>
+        <v>22.6105</v>
       </c>
       <c r="G3" t="n">
         <v>3.416844086692463e-113</v>
@@ -510,19 +510,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.2646677082932205</v>
+        <v>-0.2647</v>
       </c>
       <c r="C4" t="n">
-        <v>0.007494751020465687</v>
+        <v>0.0075</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.3504497355341742</v>
+        <v>-0.3504</v>
       </c>
       <c r="E4" t="n">
-        <v>0.009923891093305548</v>
+        <v>0.009900000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>-35.31374258737888</v>
+        <v>-35.3137</v>
       </c>
       <c r="G4" t="n">
         <v>3.613434805884537e-273</v>
@@ -535,19 +535,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.001193444128414648</v>
+        <v>-0.0012</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0005451496638546373</v>
+        <v>0.0005</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.01767857637219977</v>
+        <v>-0.0177</v>
       </c>
       <c r="E5" t="n">
-        <v>0.008075342395404379</v>
+        <v>0.0081</v>
       </c>
       <c r="F5" t="n">
-        <v>-2.189204557104665</v>
+        <v>-2.1892</v>
       </c>
       <c r="G5" t="n">
         <v>0.02858197558367184</v>
@@ -560,19 +560,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.06631146661836736</v>
+        <v>0.0663</v>
       </c>
       <c r="C6" t="n">
-        <v>0.009181824463075267</v>
+        <v>0.0092</v>
       </c>
       <c r="D6" t="n">
-        <v>0.07532570921234086</v>
+        <v>0.07530000000000001</v>
       </c>
       <c r="E6" t="n">
-        <v>0.01042998254773623</v>
+        <v>0.0104</v>
       </c>
       <c r="F6" t="n">
-        <v>7.22203597825673</v>
+        <v>7.222</v>
       </c>
       <c r="G6" t="n">
         <v>5.121491758353771e-13</v>
@@ -585,19 +585,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.09663618630069984</v>
+        <v>0.09660000000000001</v>
       </c>
       <c r="C7" t="n">
-        <v>0.009815550098897844</v>
+        <v>0.0098</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1037110872892521</v>
+        <v>0.1037</v>
       </c>
       <c r="E7" t="n">
-        <v>0.01053416336124027</v>
+        <v>0.0105</v>
       </c>
       <c r="F7" t="n">
-        <v>9.845213495629837</v>
+        <v>9.8452</v>
       </c>
       <c r="G7" t="n">
         <v>7.18864398705146e-23</v>
@@ -610,19 +610,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.06251063690323681</v>
+        <v>0.0625</v>
       </c>
       <c r="C8" t="n">
-        <v>0.009174040190048265</v>
+        <v>0.0092</v>
       </c>
       <c r="D8" t="n">
-        <v>0.06069865443742067</v>
+        <v>0.0607</v>
       </c>
       <c r="E8" t="n">
-        <v>0.008908114248663411</v>
+        <v>0.0089</v>
       </c>
       <c r="F8" t="n">
-        <v>6.813861244149176</v>
+        <v>6.8139</v>
       </c>
       <c r="G8" t="n">
         <v>9.501335183611905e-12</v>
@@ -635,19 +635,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.003383484822056926</v>
+        <v>-0.0034</v>
       </c>
       <c r="C9" t="n">
-        <v>0.008361915698620277</v>
+        <v>0.008399999999999999</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.003170577618155896</v>
+        <v>-0.0032</v>
       </c>
       <c r="E9" t="n">
-        <v>0.007835738640268037</v>
+        <v>0.0078</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.4046303435724906</v>
+        <v>-0.4046</v>
       </c>
       <c r="G9" t="n">
         <v>0.6857492507426544</v>
@@ -660,19 +660,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.1400427013417813</v>
+        <v>0.14</v>
       </c>
       <c r="C10" t="n">
-        <v>0.01438273272011647</v>
+        <v>0.0144</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1163016886957703</v>
+        <v>0.1163</v>
       </c>
       <c r="E10" t="n">
-        <v>0.01194447184596259</v>
+        <v>0.0119</v>
       </c>
       <c r="F10" t="n">
-        <v>9.736863228078347</v>
+        <v>9.7369</v>
       </c>
       <c r="G10" t="n">
         <v>2.099345818653748e-22</v>
@@ -685,19 +685,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.04398230665684229</v>
+        <v>0.044</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0105618678150626</v>
+        <v>0.0106</v>
       </c>
       <c r="D11" t="n">
-        <v>0.03609493541205414</v>
+        <v>0.0361</v>
       </c>
       <c r="E11" t="n">
-        <v>0.008667802250340367</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="F11" t="n">
-        <v>4.164254602213238</v>
+        <v>4.1643</v>
       </c>
       <c r="G11" t="n">
         <v>3.123713916089543e-05</v>
@@ -710,19 +710,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.07355837143582948</v>
+        <v>0.0736</v>
       </c>
       <c r="C12" t="n">
-        <v>0.01133029003350461</v>
+        <v>0.0113</v>
       </c>
       <c r="D12" t="n">
-        <v>0.05411987174455068</v>
+        <v>0.0541</v>
       </c>
       <c r="E12" t="n">
-        <v>0.008336153064192912</v>
+        <v>0.0083</v>
       </c>
       <c r="F12" t="n">
-        <v>6.492187862650582</v>
+        <v>6.4922</v>
       </c>
       <c r="G12" t="n">
         <v>8.459867074906337e-11</v>
@@ -735,19 +735,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.05561521477810218</v>
+        <v>0.0556</v>
       </c>
       <c r="C13" t="n">
-        <v>0.01182832483759637</v>
+        <v>0.0118</v>
       </c>
       <c r="D13" t="n">
-        <v>0.03786236654343974</v>
+        <v>0.0379</v>
       </c>
       <c r="E13" t="n">
-        <v>0.008052623232379945</v>
+        <v>0.0081</v>
       </c>
       <c r="F13" t="n">
-        <v>4.701867385424607</v>
+        <v>4.7019</v>
       </c>
       <c r="G13" t="n">
         <v>2.57792917769175e-06</v>
@@ -760,19 +760,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.04024942198362007</v>
+        <v>0.0402</v>
       </c>
       <c r="C14" t="n">
-        <v>0.0121551211910208</v>
+        <v>0.0122</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0253796190931974</v>
+        <v>0.0254</v>
       </c>
       <c r="E14" t="n">
-        <v>0.007664516175792637</v>
+        <v>0.0077</v>
       </c>
       <c r="F14" t="n">
-        <v>3.311313918725304</v>
+        <v>3.3113</v>
       </c>
       <c r="G14" t="n">
         <v>0.0009285897517735443</v>
@@ -785,19 +785,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.03020017969085996</v>
+        <v>-0.0302</v>
       </c>
       <c r="C15" t="n">
-        <v>0.00998105784781708</v>
+        <v>0.01</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.01785347061943688</v>
+        <v>-0.0179</v>
       </c>
       <c r="E15" t="n">
-        <v>0.005900512012212731</v>
+        <v>0.0059</v>
       </c>
       <c r="F15" t="n">
-        <v>-3.025749389626565</v>
+        <v>-3.0257</v>
       </c>
       <c r="G15" t="n">
         <v>0.002480177768151905</v>
@@ -810,19 +810,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.001521276948518539</v>
+        <v>-0.0015</v>
       </c>
       <c r="C16" t="n">
-        <v>0.01051982944307036</v>
+        <v>0.0105</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.0008694517702159131</v>
+        <v>-0.0009</v>
       </c>
       <c r="E16" t="n">
-        <v>0.006012372921678793</v>
+        <v>0.006</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.1446104194703116</v>
+        <v>-0.1446</v>
       </c>
       <c r="G16" t="n">
         <v>0.8850184701674246</v>
@@ -835,19 +835,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.1149745132743056</v>
+        <v>0.115</v>
       </c>
       <c r="C17" t="n">
-        <v>0.02359981280812879</v>
+        <v>0.0236</v>
       </c>
       <c r="D17" t="n">
-        <v>0.04534665603895969</v>
+        <v>0.0453</v>
       </c>
       <c r="E17" t="n">
-        <v>0.009307911497227555</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="F17" t="n">
-        <v>4.871840052676328</v>
+        <v>4.8718</v>
       </c>
       <c r="G17" t="n">
         <v>1.105636634491079e-06</v>
@@ -860,19 +860,19 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-0.06258108346606112</v>
+        <v>-0.0626</v>
       </c>
       <c r="C18" t="n">
-        <v>0.008836144308575725</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.0216514854101746</v>
+        <v>-0.0217</v>
       </c>
       <c r="E18" t="n">
-        <v>0.003057084329373726</v>
+        <v>0.0031</v>
       </c>
       <c r="F18" t="n">
-        <v>-7.082397172409738</v>
+        <v>-7.0824</v>
       </c>
       <c r="G18" t="n">
         <v>1.416818879886341e-12</v>
@@ -885,19 +885,19 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.08625824630920757</v>
+        <v>0.0863</v>
       </c>
       <c r="C19" t="n">
-        <v>0.02523616482623088</v>
+        <v>0.0252</v>
       </c>
       <c r="D19" t="n">
-        <v>0.02502470882421028</v>
+        <v>0.025</v>
       </c>
       <c r="E19" t="n">
-        <v>0.007321360028030076</v>
+        <v>0.0073</v>
       </c>
       <c r="F19" t="n">
-        <v>3.418041009921973</v>
+        <v>3.418</v>
       </c>
       <c r="G19" t="n">
         <v>0.0006307360247045329</v>
@@ -910,19 +910,19 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.05652733154884899</v>
+        <v>0.0565</v>
       </c>
       <c r="C20" t="n">
-        <v>0.03079923924048143</v>
+        <v>0.0308</v>
       </c>
       <c r="D20" t="n">
-        <v>0.01136717701512804</v>
+        <v>0.0114</v>
       </c>
       <c r="E20" t="n">
-        <v>0.00619347127814242</v>
+        <v>0.0062</v>
       </c>
       <c r="F20" t="n">
-        <v>1.835348305439684</v>
+        <v>1.8353</v>
       </c>
       <c r="G20" t="n">
         <v>0.06645409798580651</v>
@@ -935,19 +935,19 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-0.3081649680877036</v>
+        <v>-0.3082</v>
       </c>
       <c r="C21" t="n">
-        <v>0.04245361604253767</v>
+        <v>0.0425</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.04386480052077236</v>
+        <v>-0.0439</v>
       </c>
       <c r="E21" t="n">
-        <v>0.006042930222235349</v>
+        <v>0.006</v>
       </c>
       <c r="F21" t="n">
-        <v>-7.258862655631702</v>
+        <v>-7.2589</v>
       </c>
       <c r="G21" t="n">
         <v>3.903585811780023e-13</v>
@@ -960,19 +960,19 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>-0.1311089914432668</v>
+        <v>-0.1311</v>
       </c>
       <c r="C22" t="n">
-        <v>0.006022886358007171</v>
+        <v>0.006</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.1742917649144759</v>
+        <v>-0.1743</v>
       </c>
       <c r="E22" t="n">
-        <v>0.008006617102768506</v>
+        <v>0.008</v>
       </c>
       <c r="F22" t="n">
-        <v>-21.76846509298037</v>
+        <v>-21.7685</v>
       </c>
       <c r="G22" t="n">
         <v>4.618387003790065e-105</v>
@@ -985,19 +985,19 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-0.1107515140736464</v>
+        <v>-0.1108</v>
       </c>
       <c r="C23" t="n">
-        <v>0.007485696856691884</v>
+        <v>0.0075</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.1151570868563532</v>
+        <v>-0.1152</v>
       </c>
       <c r="E23" t="n">
-        <v>0.007783469601446468</v>
+        <v>0.0078</v>
       </c>
       <c r="F23" t="n">
-        <v>-14.79508403745196</v>
+        <v>-14.7951</v>
       </c>
       <c r="G23" t="n">
         <v>1.575873980804803e-49</v>
@@ -1010,19 +1010,19 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>-0.2372773237589519</v>
+        <v>-0.2373</v>
       </c>
       <c r="C24" t="n">
-        <v>0.009452746660971361</v>
+        <v>0.0095</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.1722802254946329</v>
+        <v>-0.1723</v>
       </c>
       <c r="E24" t="n">
-        <v>0.006863366884355901</v>
+        <v>0.0069</v>
       </c>
       <c r="F24" t="n">
-        <v>-25.10141573333664</v>
+        <v>-25.1014</v>
       </c>
       <c r="G24" t="n">
         <v>4.799422352546218e-139</v>
@@ -1035,19 +1035,19 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>-0.04320650554590563</v>
+        <v>-0.0432</v>
       </c>
       <c r="C25" t="n">
-        <v>0.008266537090080094</v>
+        <v>0.0083</v>
       </c>
       <c r="D25" t="n">
-        <v>-0.04992295848619177</v>
+        <v>-0.0499</v>
       </c>
       <c r="E25" t="n">
-        <v>0.009551570597028778</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="F25" t="n">
-        <v>-5.22667533878893</v>
+        <v>-5.2267</v>
       </c>
       <c r="G25" t="n">
         <v>1.725851529309045e-07</v>
@@ -1060,19 +1060,19 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>-0.1595856016157796</v>
+        <v>-0.1596</v>
       </c>
       <c r="C26" t="n">
-        <v>0.006430429664423285</v>
+        <v>0.0064</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.1613499190370889</v>
+        <v>-0.1613</v>
       </c>
       <c r="E26" t="n">
-        <v>0.006501522037222436</v>
+        <v>0.0065</v>
       </c>
       <c r="F26" t="n">
-        <v>-24.81725326982363</v>
+        <v>-24.8173</v>
       </c>
       <c r="G26" t="n">
         <v>5.839207849537465e-136</v>
@@ -1136,15 +1136,15 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2777986468582379</v>
+        <v>0.2778</v>
       </c>
       <c r="C2" t="n">
-        <v>0.009045722481464413</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>30.71049851766678</v>
+        <v>30.7105</v>
       </c>
       <c r="G2" t="n">
         <v>4.121846448096214e-207</v>
@@ -1157,19 +1157,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.07839545140456043</v>
+        <v>0.0784</v>
       </c>
       <c r="C3" t="n">
-        <v>0.003855048023438303</v>
+        <v>0.0039</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2573863037393153</v>
+        <v>0.2574</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0126568129108651</v>
+        <v>0.0127</v>
       </c>
       <c r="F3" t="n">
-        <v>20.33579113098566</v>
+        <v>20.3358</v>
       </c>
       <c r="G3" t="n">
         <v>6.203109040878432e-92</v>
@@ -1182,19 +1182,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.1548845476955757</v>
+        <v>-0.1549</v>
       </c>
       <c r="C4" t="n">
-        <v>0.005913038048582205</v>
+        <v>0.0059</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.2965496231808294</v>
+        <v>-0.2965</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01132139539579809</v>
+        <v>0.0113</v>
       </c>
       <c r="F4" t="n">
-        <v>-26.19373432455978</v>
+        <v>-26.1937</v>
       </c>
       <c r="G4" t="n">
         <v>3.13217078813274e-151</v>
@@ -1207,19 +1207,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.001315990753542443</v>
+        <v>-0.0013</v>
       </c>
       <c r="C5" t="n">
-        <v>0.000465485405620212</v>
+        <v>0.0005</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.02598201546251751</v>
+        <v>-0.026</v>
       </c>
       <c r="E5" t="n">
-        <v>0.009190223391649778</v>
+        <v>0.0092</v>
       </c>
       <c r="F5" t="n">
-        <v>-2.827136442202779</v>
+        <v>-2.8271</v>
       </c>
       <c r="G5" t="n">
         <v>0.004696631178074946</v>
@@ -1232,19 +1232,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.0632990336894094</v>
+        <v>0.0633</v>
       </c>
       <c r="C6" t="n">
-        <v>0.00923940306674109</v>
+        <v>0.0092</v>
       </c>
       <c r="D6" t="n">
-        <v>0.09855164103476707</v>
+        <v>0.09859999999999999</v>
       </c>
       <c r="E6" t="n">
-        <v>0.01438502740621363</v>
+        <v>0.0144</v>
       </c>
       <c r="F6" t="n">
-        <v>6.850987367059</v>
+        <v>6.851</v>
       </c>
       <c r="G6" t="n">
         <v>7.334199362201158e-12</v>
@@ -1257,19 +1257,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.08066712117979756</v>
+        <v>0.08069999999999999</v>
       </c>
       <c r="C7" t="n">
-        <v>0.009466039941280693</v>
+        <v>0.0095</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1208146849730236</v>
+        <v>0.1208</v>
       </c>
       <c r="E7" t="n">
-        <v>0.01417723375672294</v>
+        <v>0.0142</v>
       </c>
       <c r="F7" t="n">
-        <v>8.521738940484951</v>
+        <v>8.521699999999999</v>
       </c>
       <c r="G7" t="n">
         <v>1.571753521963822e-17</v>
@@ -1282,19 +1282,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.07723327199807399</v>
+        <v>0.0772</v>
       </c>
       <c r="C8" t="n">
-        <v>0.009720868605305385</v>
+        <v>0.0097</v>
       </c>
       <c r="D8" t="n">
-        <v>0.09607930905177713</v>
+        <v>0.0961</v>
       </c>
       <c r="E8" t="n">
-        <v>0.01209290134702755</v>
+        <v>0.0121</v>
       </c>
       <c r="F8" t="n">
-        <v>7.94509988088124</v>
+        <v>7.9451</v>
       </c>
       <c r="G8" t="n">
         <v>1.940343772614067e-15</v>
@@ -1307,19 +1307,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.03430475571610891</v>
+        <v>0.0343</v>
       </c>
       <c r="C9" t="n">
-        <v>0.009595090718052772</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="D9" t="n">
-        <v>0.03576095157738726</v>
+        <v>0.0358</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0100023908459956</v>
+        <v>0.01</v>
       </c>
       <c r="F9" t="n">
-        <v>3.575240372825857</v>
+        <v>3.5752</v>
       </c>
       <c r="G9" t="n">
         <v>0.0003499062625434746</v>
@@ -1332,19 +1332,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.1111827367386595</v>
+        <v>0.1112</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0126135091700904</v>
+        <v>0.0126</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1356695076578593</v>
+        <v>0.1357</v>
       </c>
       <c r="E10" t="n">
-        <v>0.01539149538085647</v>
+        <v>0.0154</v>
       </c>
       <c r="F10" t="n">
-        <v>8.814576121472996</v>
+        <v>8.8146</v>
       </c>
       <c r="G10" t="n">
         <v>1.201387264815336e-18</v>
@@ -1357,19 +1357,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.02443124612557207</v>
+        <v>0.0244</v>
       </c>
       <c r="C11" t="n">
-        <v>0.009557662671892266</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="D11" t="n">
-        <v>0.02943995140631993</v>
+        <v>0.0294</v>
       </c>
       <c r="E11" t="n">
-        <v>0.01151710081312595</v>
+        <v>0.0115</v>
       </c>
       <c r="F11" t="n">
-        <v>2.556194643426882</v>
+        <v>2.5562</v>
       </c>
       <c r="G11" t="n">
         <v>0.01058239055606917</v>
@@ -1382,19 +1382,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.07756457838091581</v>
+        <v>0.0776</v>
       </c>
       <c r="C12" t="n">
-        <v>0.01107869663848694</v>
+        <v>0.0111</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0748063070607778</v>
+        <v>0.07480000000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>0.01068472748606818</v>
+        <v>0.0107</v>
       </c>
       <c r="F12" t="n">
-        <v>7.001236780097365</v>
+        <v>7.0012</v>
       </c>
       <c r="G12" t="n">
         <v>2.537127339931194e-12</v>
@@ -1407,19 +1407,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.03851234493399321</v>
+        <v>0.0385</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0100209068257704</v>
+        <v>0.01</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0390369970610609</v>
+        <v>0.039</v>
       </c>
       <c r="E13" t="n">
-        <v>0.01015742123667679</v>
+        <v>0.0102</v>
       </c>
       <c r="F13" t="n">
-        <v>3.843199582991075</v>
+        <v>3.8432</v>
       </c>
       <c r="G13" t="n">
         <v>0.0001214406303753483</v>
@@ -1432,19 +1432,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.05608239709869824</v>
+        <v>0.0561</v>
       </c>
       <c r="C14" t="n">
-        <v>0.01177342940935744</v>
+        <v>0.0118</v>
       </c>
       <c r="D14" t="n">
-        <v>0.04713653148156568</v>
+        <v>0.0471</v>
       </c>
       <c r="E14" t="n">
-        <v>0.009895415579749701</v>
+        <v>0.009900000000000001</v>
       </c>
       <c r="F14" t="n">
-        <v>4.763471640142876</v>
+        <v>4.7635</v>
       </c>
       <c r="G14" t="n">
         <v>1.902903654966833e-06</v>
@@ -1457,19 +1457,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.02742887116376902</v>
+        <v>-0.0274</v>
       </c>
       <c r="C15" t="n">
-        <v>0.01057591723238545</v>
+        <v>0.0106</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.01874368335421085</v>
+        <v>-0.0187</v>
       </c>
       <c r="E15" t="n">
-        <v>0.007227116369485166</v>
+        <v>0.0072</v>
       </c>
       <c r="F15" t="n">
-        <v>-2.593521730652038</v>
+        <v>-2.5935</v>
       </c>
       <c r="G15" t="n">
         <v>0.009499853553076362</v>
@@ -1482,19 +1482,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.005010339418654501</v>
+        <v>0.005</v>
       </c>
       <c r="C16" t="n">
-        <v>0.0101869734449156</v>
+        <v>0.0102</v>
       </c>
       <c r="D16" t="n">
-        <v>0.003927189110710777</v>
+        <v>0.0039</v>
       </c>
       <c r="E16" t="n">
-        <v>0.007984722758506415</v>
+        <v>0.008</v>
       </c>
       <c r="F16" t="n">
-        <v>0.4918378795966334</v>
+        <v>0.4918</v>
       </c>
       <c r="G16" t="n">
         <v>0.6228339559200247</v>
@@ -1507,19 +1507,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.06597891720411807</v>
+        <v>0.066</v>
       </c>
       <c r="C17" t="n">
-        <v>0.01868459494621359</v>
+        <v>0.0187</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0372164344452271</v>
+        <v>0.0372</v>
       </c>
       <c r="E17" t="n">
-        <v>0.01053933638832099</v>
+        <v>0.0105</v>
       </c>
       <c r="F17" t="n">
-        <v>3.531193338365016</v>
+        <v>3.5312</v>
       </c>
       <c r="G17" t="n">
         <v>0.0004136892471294721</v>
@@ -1532,19 +1532,19 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.07422412464631249</v>
+        <v>0.0742</v>
       </c>
       <c r="C18" t="n">
-        <v>0.0253455807765246</v>
+        <v>0.0253</v>
       </c>
       <c r="D18" t="n">
-        <v>0.02774863339095885</v>
+        <v>0.0277</v>
       </c>
       <c r="E18" t="n">
-        <v>0.009475426384616258</v>
+        <v>0.0095</v>
       </c>
       <c r="F18" t="n">
-        <v>2.92848387656833</v>
+        <v>2.9285</v>
       </c>
       <c r="G18" t="n">
         <v>0.003406194983078177</v>
@@ -1557,19 +1557,19 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.03231082833638427</v>
+        <v>0.0323</v>
       </c>
       <c r="C19" t="n">
-        <v>0.02267244677812823</v>
+        <v>0.0227</v>
       </c>
       <c r="D19" t="n">
-        <v>0.008785027514731489</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="E19" t="n">
-        <v>0.006164437095159622</v>
+        <v>0.0062</v>
       </c>
       <c r="F19" t="n">
-        <v>1.425114309566007</v>
+        <v>1.4251</v>
       </c>
       <c r="G19" t="n">
         <v>0.1541241609055243</v>
@@ -1582,19 +1582,19 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-0.06124395690136044</v>
+        <v>-0.0612</v>
       </c>
       <c r="C20" t="n">
-        <v>0.005186959996277839</v>
+        <v>0.0052</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.1073858247555929</v>
+        <v>-0.1074</v>
       </c>
       <c r="E20" t="n">
-        <v>0.009094872463444467</v>
+        <v>0.0091</v>
       </c>
       <c r="F20" t="n">
-        <v>-11.80729308599046</v>
+        <v>-11.8073</v>
       </c>
       <c r="G20" t="n">
         <v>3.578989638699906e-32</v>
@@ -1607,19 +1607,19 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-0.0435226201930169</v>
+        <v>-0.0435</v>
       </c>
       <c r="C21" t="n">
-        <v>0.006012887130669324</v>
+        <v>0.006</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.06562345209408321</v>
+        <v>-0.06560000000000001</v>
       </c>
       <c r="E21" t="n">
-        <v>0.009066237483328689</v>
+        <v>0.0091</v>
       </c>
       <c r="F21" t="n">
-        <v>-7.23822337709043</v>
+        <v>-7.2382</v>
       </c>
       <c r="G21" t="n">
         <v>4.546002757444119e-13</v>
@@ -1632,19 +1632,19 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>-0.1572942281385584</v>
+        <v>-0.1573</v>
       </c>
       <c r="C22" t="n">
-        <v>0.01197350538976417</v>
+        <v>0.012</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.1115202358532186</v>
+        <v>-0.1115</v>
       </c>
       <c r="E22" t="n">
-        <v>0.008489110890197748</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="F22" t="n">
-        <v>-13.1368570037163</v>
+        <v>-13.1369</v>
       </c>
       <c r="G22" t="n">
         <v>2.024629328319839e-39</v>
@@ -1657,19 +1657,19 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.008906718157930458</v>
+        <v>0.0089</v>
       </c>
       <c r="C23" t="n">
-        <v>0.006728659038823263</v>
+        <v>0.0067</v>
       </c>
       <c r="D23" t="n">
-        <v>0.01514732354565864</v>
+        <v>0.0151</v>
       </c>
       <c r="E23" t="n">
-        <v>0.01144317959569954</v>
+        <v>0.0114</v>
       </c>
       <c r="F23" t="n">
-        <v>1.323698839031693</v>
+        <v>1.3237</v>
       </c>
       <c r="G23" t="n">
         <v>0.1856030841934638</v>
@@ -1682,19 +1682,19 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>-0.1039332756087135</v>
+        <v>-0.1039</v>
       </c>
       <c r="C24" t="n">
-        <v>0.00650955666450826</v>
+        <v>0.0065</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.1057551060924098</v>
+        <v>-0.1058</v>
       </c>
       <c r="E24" t="n">
-        <v>0.006623661687151804</v>
+        <v>0.0066</v>
       </c>
       <c r="F24" t="n">
-        <v>-15.96626021790145</v>
+        <v>-15.9663</v>
       </c>
       <c r="G24" t="n">
         <v>2.195617844741011e-57</v>
@@ -1758,15 +1758,15 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1269118006192248</v>
+        <v>0.1269</v>
       </c>
       <c r="C2" t="n">
-        <v>0.005568671878613018</v>
+        <v>0.0056</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>22.79031758122452</v>
+        <v>22.7903</v>
       </c>
       <c r="G2" t="n">
         <v>5.719919393903775e-115</v>
@@ -1779,19 +1779,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.01271564074863031</v>
+        <v>0.0127</v>
       </c>
       <c r="C3" t="n">
-        <v>0.002573760272582135</v>
+        <v>0.0026</v>
       </c>
       <c r="D3" t="n">
-        <v>0.07381207773740775</v>
+        <v>0.0738</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01494022968034449</v>
+        <v>0.0149</v>
       </c>
       <c r="F3" t="n">
-        <v>4.940491499572837</v>
+        <v>4.9405</v>
       </c>
       <c r="G3" t="n">
         <v>7.792589020641442e-07</v>
@@ -1804,19 +1804,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.01779226790884811</v>
+        <v>-0.0178</v>
       </c>
       <c r="C4" t="n">
-        <v>0.003742112828306235</v>
+        <v>0.0037</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.07491491964331772</v>
+        <v>-0.07489999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01575628712792576</v>
+        <v>0.0158</v>
       </c>
       <c r="F4" t="n">
-        <v>-4.754604878362604</v>
+        <v>-4.7546</v>
       </c>
       <c r="G4" t="n">
         <v>1.988349022704924e-06</v>
@@ -1829,19 +1829,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.004386187369941517</v>
+        <v>-0.0044</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0003521984132819927</v>
+        <v>0.0004</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.200341633006248</v>
+        <v>-0.2003</v>
       </c>
       <c r="E5" t="n">
-        <v>0.01608686526769709</v>
+        <v>0.0161</v>
       </c>
       <c r="F5" t="n">
-        <v>-12.45373972321009</v>
+        <v>-12.4537</v>
       </c>
       <c r="G5" t="n">
         <v>1.334427727785046e-35</v>
@@ -1854,19 +1854,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.02069278390147021</v>
+        <v>-0.0207</v>
       </c>
       <c r="C6" t="n">
-        <v>0.005029681665980132</v>
+        <v>0.005</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.0747562439595806</v>
+        <v>-0.07480000000000001</v>
       </c>
       <c r="E6" t="n">
-        <v>0.01817059084226583</v>
+        <v>0.0182</v>
       </c>
       <c r="F6" t="n">
-        <v>-4.114133910587722</v>
+        <v>-4.1141</v>
       </c>
       <c r="G6" t="n">
         <v>3.886357916280625e-05</v>
@@ -1879,19 +1879,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.001357760895420551</v>
+        <v>-0.0014</v>
       </c>
       <c r="C7" t="n">
-        <v>0.006846145983917602</v>
+        <v>0.0068</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.003909026135805856</v>
+        <v>-0.0039</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0197102182504579</v>
+        <v>0.0197</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1983248529333279</v>
+        <v>-0.1983</v>
       </c>
       <c r="G7" t="n">
         <v>0.8427909080393092</v>
@@ -1904,19 +1904,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-0.02780300856431317</v>
+        <v>-0.0278</v>
       </c>
       <c r="C8" t="n">
-        <v>0.005886621935506595</v>
+        <v>0.0059</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.08276920258465133</v>
+        <v>-0.0828</v>
       </c>
       <c r="E8" t="n">
-        <v>0.01752439856975004</v>
+        <v>0.0175</v>
       </c>
       <c r="F8" t="n">
-        <v>-4.723083776896312</v>
+        <v>-4.7231</v>
       </c>
       <c r="G8" t="n">
         <v>2.322951006754869e-06</v>
@@ -1929,19 +1929,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.05661962386928919</v>
+        <v>-0.0566</v>
       </c>
       <c r="C9" t="n">
-        <v>0.004404107065777839</v>
+        <v>0.0044</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.1982238500801443</v>
+        <v>-0.1982</v>
       </c>
       <c r="E9" t="n">
-        <v>0.01541866581026813</v>
+        <v>0.0154</v>
       </c>
       <c r="F9" t="n">
-        <v>-12.85609614472195</v>
+        <v>-12.8561</v>
       </c>
       <c r="G9" t="n">
         <v>7.949098793573911e-38</v>
@@ -1954,19 +1954,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.03713303717540821</v>
+        <v>-0.0371</v>
       </c>
       <c r="C10" t="n">
-        <v>0.005995157129898481</v>
+        <v>0.006</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.09049667849481709</v>
+        <v>-0.0905</v>
       </c>
       <c r="E10" t="n">
-        <v>0.01461075765894091</v>
+        <v>0.0146</v>
       </c>
       <c r="F10" t="n">
-        <v>-6.193838855402444</v>
+        <v>-6.1938</v>
       </c>
       <c r="G10" t="n">
         <v>5.871625820920273e-10</v>
@@ -1979,19 +1979,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-0.06794980909126752</v>
+        <v>-0.0679</v>
       </c>
       <c r="C11" t="n">
-        <v>0.006081853727832097</v>
+        <v>0.0061</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.122865943855642</v>
+        <v>-0.1229</v>
       </c>
       <c r="E11" t="n">
-        <v>0.01099712727166555</v>
+        <v>0.011</v>
       </c>
       <c r="F11" t="n">
-        <v>-11.17254905035155</v>
+        <v>-11.1725</v>
       </c>
       <c r="G11" t="n">
         <v>5.556307084838132e-29</v>
@@ -2004,19 +2004,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.03424450623555214</v>
+        <v>-0.0342</v>
       </c>
       <c r="C12" t="n">
-        <v>0.007262890533516435</v>
+        <v>0.0073</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.07282455611289536</v>
+        <v>-0.0728</v>
       </c>
       <c r="E12" t="n">
-        <v>0.01544530312575424</v>
+        <v>0.0154</v>
       </c>
       <c r="F12" t="n">
-        <v>-4.714996884163716</v>
+        <v>-4.715</v>
       </c>
       <c r="G12" t="n">
         <v>2.417144481668843e-06</v>
@@ -2029,19 +2029,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.03363803609019785</v>
+        <v>-0.0336</v>
       </c>
       <c r="C13" t="n">
-        <v>0.009118255449115851</v>
+        <v>0.0091</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.05392952160092151</v>
+        <v>-0.0539</v>
       </c>
       <c r="E13" t="n">
-        <v>0.01461866420760241</v>
+        <v>0.0146</v>
       </c>
       <c r="F13" t="n">
-        <v>-3.689086830031675</v>
+        <v>-3.6891</v>
       </c>
       <c r="G13" t="n">
         <v>0.0002250604045411201</v>
@@ -2054,19 +2054,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.02815760575532223</v>
+        <v>-0.0282</v>
       </c>
       <c r="C14" t="n">
-        <v>0.006064204594641256</v>
+        <v>0.0061</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.06799376778499104</v>
+        <v>-0.068</v>
       </c>
       <c r="E14" t="n">
-        <v>0.01464357881105629</v>
+        <v>0.0146</v>
       </c>
       <c r="F14" t="n">
-        <v>-4.643247983454287</v>
+        <v>-4.6432</v>
       </c>
       <c r="G14" t="n">
         <v>3.429742796471264e-06</v>
@@ -2079,19 +2079,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.0093470351045024</v>
+        <v>-0.009299999999999999</v>
       </c>
       <c r="C15" t="n">
-        <v>0.00837661908171846</v>
+        <v>0.008399999999999999</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.01773123291957474</v>
+        <v>-0.0177</v>
       </c>
       <c r="E15" t="n">
-        <v>0.01589036334580144</v>
+        <v>0.0159</v>
       </c>
       <c r="F15" t="n">
-        <v>-1.115848173746115</v>
+        <v>-1.1158</v>
       </c>
       <c r="G15" t="n">
         <v>0.2644871290746181</v>
@@ -2104,19 +2104,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.03402195088972423</v>
+        <v>-0.034</v>
       </c>
       <c r="C16" t="n">
-        <v>0.008563905267768342</v>
+        <v>0.0086</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.04765711590058416</v>
+        <v>-0.0477</v>
       </c>
       <c r="E16" t="n">
-        <v>0.01199610884250992</v>
+        <v>0.012</v>
       </c>
       <c r="F16" t="n">
-        <v>-3.972714529873586</v>
+        <v>-3.9727</v>
       </c>
       <c r="G16" t="n">
         <v>7.105818977226174e-05</v>
@@ -2129,19 +2129,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-0.03146750762450962</v>
+        <v>-0.0315</v>
       </c>
       <c r="C17" t="n">
-        <v>0.006904683022540094</v>
+        <v>0.0069</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.04006098487052581</v>
+        <v>-0.0401</v>
       </c>
       <c r="E17" t="n">
-        <v>0.008790286329709462</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="F17" t="n">
-        <v>-4.557415238583009</v>
+        <v>-4.5574</v>
       </c>
       <c r="G17" t="n">
         <v>5.178697854291059e-06</v>
@@ -2154,19 +2154,19 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-0.04897591731650213</v>
+        <v>-0.049</v>
       </c>
       <c r="C18" t="n">
-        <v>0.004395934670633928</v>
+        <v>0.0044</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.08878093660926895</v>
+        <v>-0.0888</v>
       </c>
       <c r="E18" t="n">
-        <v>0.007968716436895356</v>
+        <v>0.008</v>
       </c>
       <c r="F18" t="n">
-        <v>-11.14118406801515</v>
+        <v>-11.1412</v>
       </c>
       <c r="G18" t="n">
         <v>7.906114396722562e-29</v>
@@ -2179,19 +2179,19 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.02443991878371804</v>
+        <v>0.0244</v>
       </c>
       <c r="C19" t="n">
-        <v>0.01657393499568657</v>
+        <v>0.0166</v>
       </c>
       <c r="D19" t="n">
-        <v>0.02290277790027005</v>
+        <v>0.0229</v>
       </c>
       <c r="E19" t="n">
-        <v>0.01553152264943722</v>
+        <v>0.0155</v>
       </c>
       <c r="F19" t="n">
-        <v>1.474599652410765</v>
+        <v>1.4746</v>
       </c>
       <c r="G19" t="n">
         <v>0.1403202084202728</v>
@@ -2204,19 +2204,19 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.02900195765188757</v>
+        <v>0.029</v>
       </c>
       <c r="C20" t="n">
-        <v>0.02350204269450779</v>
+        <v>0.0235</v>
       </c>
       <c r="D20" t="n">
-        <v>0.01926081844483624</v>
+        <v>0.0193</v>
       </c>
       <c r="E20" t="n">
-        <v>0.01560820765463889</v>
+        <v>0.0156</v>
       </c>
       <c r="F20" t="n">
-        <v>1.234018592718541</v>
+        <v>1.234</v>
       </c>
       <c r="G20" t="n">
         <v>0.2171959761181209</v>
@@ -2229,19 +2229,19 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-0.004056156409897579</v>
+        <v>-0.0041</v>
       </c>
       <c r="C21" t="n">
-        <v>0.01656033922952283</v>
+        <v>0.0166</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.003045753955177786</v>
+        <v>-0.003</v>
       </c>
       <c r="E21" t="n">
-        <v>0.01243510200551626</v>
+        <v>0.0124</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.2449319638734509</v>
+        <v>-0.2449</v>
       </c>
       <c r="G21" t="n">
         <v>0.806509111750946</v>
@@ -2254,19 +2254,19 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.002306186679775542</v>
+        <v>0.0023</v>
       </c>
       <c r="C22" t="n">
-        <v>0.003778413852833541</v>
+        <v>0.0038</v>
       </c>
       <c r="D22" t="n">
-        <v>0.00988637677543085</v>
+        <v>0.009900000000000001</v>
       </c>
       <c r="E22" t="n">
-        <v>0.01619765793038723</v>
+        <v>0.0162</v>
       </c>
       <c r="F22" t="n">
-        <v>0.6103584121803033</v>
+        <v>0.6104000000000001</v>
       </c>
       <c r="G22" t="n">
         <v>0.5416244107718886</v>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-0.02415223603248558</v>
+        <v>-0.0242</v>
       </c>
       <c r="C23" t="n">
-        <v>0.005305977150646527</v>
+        <v>0.0053</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.0589377945754163</v>
+        <v>-0.0589</v>
       </c>
       <c r="E23" t="n">
-        <v>0.01294797677970831</v>
+        <v>0.0129</v>
       </c>
       <c r="F23" t="n">
-        <v>-4.55189220510357</v>
+        <v>-4.5519</v>
       </c>
       <c r="G23" t="n">
         <v>5.316557525235557e-06</v>
@@ -2304,19 +2304,19 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>-0.07133108183472997</v>
+        <v>-0.0713</v>
       </c>
       <c r="C24" t="n">
-        <v>0.003404646192628418</v>
+        <v>0.0034</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.2002510515689492</v>
+        <v>-0.2003</v>
       </c>
       <c r="E24" t="n">
-        <v>0.009558021030351319</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="F24" t="n">
-        <v>-20.95109970286273</v>
+        <v>-20.9511</v>
       </c>
       <c r="G24" t="n">
         <v>1.833481854511251e-97</v>
@@ -2329,19 +2329,19 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>-0.01783240154662832</v>
+        <v>-0.0178</v>
       </c>
       <c r="C25" t="n">
-        <v>0.002975924990689684</v>
+        <v>0.003</v>
       </c>
       <c r="D25" t="n">
-        <v>-0.07627550717530844</v>
+        <v>-0.07630000000000001</v>
       </c>
       <c r="E25" t="n">
-        <v>0.01272908684716384</v>
+        <v>0.0127</v>
       </c>
       <c r="F25" t="n">
-        <v>-5.992221444565236</v>
+        <v>-5.9922</v>
       </c>
       <c r="G25" t="n">
         <v>2.069937966897287e-09</v>
@@ -2405,15 +2405,15 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2223184151331574</v>
+        <v>0.2223</v>
       </c>
       <c r="C2" t="n">
-        <v>0.007954534617253751</v>
+        <v>0.008</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>27.94863883688916</v>
+        <v>27.9486</v>
       </c>
       <c r="G2" t="n">
         <v>6.848253084229291e-172</v>
@@ -2426,19 +2426,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.05791629399901178</v>
+        <v>0.0579</v>
       </c>
       <c r="C3" t="n">
-        <v>0.003325955595044214</v>
+        <v>0.0033</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2254799177218793</v>
+        <v>0.2255</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01294862191855697</v>
+        <v>0.0129</v>
       </c>
       <c r="F3" t="n">
-        <v>17.41342971785583</v>
+        <v>17.4134</v>
       </c>
       <c r="G3" t="n">
         <v>6.52548235122811e-68</v>
@@ -2451,19 +2451,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.116495056224795</v>
+        <v>-0.1165</v>
       </c>
       <c r="C4" t="n">
-        <v>0.005260636528222098</v>
+        <v>0.0053</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.2631166039349796</v>
+        <v>-0.2631</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01188171294729581</v>
+        <v>0.0119</v>
       </c>
       <c r="F4" t="n">
-        <v>-22.14466929996512</v>
+        <v>-22.1447</v>
       </c>
       <c r="G4" t="n">
         <v>1.174196130163128e-108</v>
@@ -2476,19 +2476,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.005547012012503857</v>
+        <v>0.0055</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0004839974841475091</v>
+        <v>0.0005</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1241219899536324</v>
+        <v>0.1241</v>
       </c>
       <c r="E5" t="n">
-        <v>0.01083010650229752</v>
+        <v>0.0108</v>
       </c>
       <c r="F5" t="n">
-        <v>11.4608281947459</v>
+        <v>11.4608</v>
       </c>
       <c r="G5" t="n">
         <v>2.07520829055946e-30</v>
@@ -2501,19 +2501,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.06248938180439636</v>
+        <v>0.0625</v>
       </c>
       <c r="C6" t="n">
-        <v>0.00790846700924375</v>
+        <v>0.007900000000000001</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1144776488886845</v>
+        <v>0.1145</v>
       </c>
       <c r="E6" t="n">
-        <v>0.01448794472580711</v>
+        <v>0.0145</v>
       </c>
       <c r="F6" t="n">
-        <v>7.901579627424143</v>
+        <v>7.9016</v>
       </c>
       <c r="G6" t="n">
         <v>2.753908328349476e-15</v>
@@ -2526,19 +2526,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.07112519003058633</v>
+        <v>0.0711</v>
       </c>
       <c r="C7" t="n">
-        <v>0.008784942602163932</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="D7" t="n">
-        <v>0.122131774420529</v>
+        <v>0.1221</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0150849597410339</v>
+        <v>0.0151</v>
       </c>
       <c r="F7" t="n">
-        <v>8.096261210980089</v>
+        <v>8.096299999999999</v>
       </c>
       <c r="G7" t="n">
         <v>5.667406196789904e-16</v>
@@ -2551,19 +2551,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.06742474315306365</v>
+        <v>0.0674</v>
       </c>
       <c r="C8" t="n">
-        <v>0.008177551961045871</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="D8" t="n">
-        <v>0.09478414953304827</v>
+        <v>0.0948</v>
       </c>
       <c r="E8" t="n">
-        <v>0.01149581402379914</v>
+        <v>0.0115</v>
       </c>
       <c r="F8" t="n">
-        <v>8.245101159154279</v>
+        <v>8.245100000000001</v>
       </c>
       <c r="G8" t="n">
         <v>1.650205533892556e-16</v>
@@ -2576,19 +2576,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.04473164934305855</v>
+        <v>0.0447</v>
       </c>
       <c r="C9" t="n">
-        <v>0.007941617831481491</v>
+        <v>0.007900000000000001</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0553200161215196</v>
+        <v>0.0553</v>
       </c>
       <c r="E9" t="n">
-        <v>0.009821467192035898</v>
+        <v>0.0098</v>
       </c>
       <c r="F9" t="n">
-        <v>5.632561310837335</v>
+        <v>5.6326</v>
       </c>
       <c r="G9" t="n">
         <v>1.775526925826283e-08</v>
@@ -2601,19 +2601,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.1096184412738307</v>
+        <v>0.1096</v>
       </c>
       <c r="C10" t="n">
-        <v>0.01039666413156494</v>
+        <v>0.0104</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1579829814346467</v>
+        <v>0.158</v>
       </c>
       <c r="E10" t="n">
-        <v>0.01498375617635603</v>
+        <v>0.015</v>
       </c>
       <c r="F10" t="n">
-        <v>10.54361667229607</v>
+        <v>10.5436</v>
       </c>
       <c r="G10" t="n">
         <v>5.436701966806563e-26</v>
@@ -2626,19 +2626,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.06243000601204574</v>
+        <v>0.0624</v>
       </c>
       <c r="C11" t="n">
-        <v>0.008170948514893544</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="D11" t="n">
-        <v>0.08835295873157133</v>
+        <v>0.08840000000000001</v>
       </c>
       <c r="E11" t="n">
-        <v>0.01156378996335334</v>
+        <v>0.0116</v>
       </c>
       <c r="F11" t="n">
-        <v>7.640484565317214</v>
+        <v>7.6405</v>
       </c>
       <c r="G11" t="n">
         <v>2.16405738727976e-14</v>
@@ -2651,19 +2651,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.07535407603663703</v>
+        <v>0.07539999999999999</v>
       </c>
       <c r="C12" t="n">
-        <v>0.01029754399503835</v>
+        <v>0.0103</v>
       </c>
       <c r="D12" t="n">
-        <v>0.08287901105849291</v>
+        <v>0.0829</v>
       </c>
       <c r="E12" t="n">
-        <v>0.01132586725932588</v>
+        <v>0.0113</v>
       </c>
       <c r="F12" t="n">
-        <v>7.317674590460094</v>
+        <v>7.3177</v>
       </c>
       <c r="G12" t="n">
         <v>2.523047702038281e-13</v>
@@ -2676,19 +2676,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.05641304178896852</v>
+        <v>0.0564</v>
       </c>
       <c r="C13" t="n">
-        <v>0.008559940075658249</v>
+        <v>0.0086</v>
       </c>
       <c r="D13" t="n">
-        <v>0.06676359191489156</v>
+        <v>0.0668</v>
       </c>
       <c r="E13" t="n">
-        <v>0.01013050046414848</v>
+        <v>0.0101</v>
       </c>
       <c r="F13" t="n">
-        <v>6.590354756032615</v>
+        <v>6.5904</v>
       </c>
       <c r="G13" t="n">
         <v>4.387768640253819e-11</v>
@@ -2701,19 +2701,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.03244946472807977</v>
+        <v>0.0324</v>
       </c>
       <c r="C14" t="n">
-        <v>0.009013322180690205</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="D14" t="n">
-        <v>0.03223605229533273</v>
+        <v>0.0322</v>
       </c>
       <c r="E14" t="n">
-        <v>0.008954043698600193</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="F14" t="n">
-        <v>3.600166961478227</v>
+        <v>3.6002</v>
       </c>
       <c r="G14" t="n">
         <v>0.0003180129136090101</v>
@@ -2726,19 +2726,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.01060733010991921</v>
+        <v>0.0106</v>
       </c>
       <c r="C15" t="n">
-        <v>0.008376711420939504</v>
+        <v>0.008399999999999999</v>
       </c>
       <c r="D15" t="n">
-        <v>0.009314668233806809</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="E15" t="n">
-        <v>0.007355883805617339</v>
+        <v>0.0074</v>
       </c>
       <c r="F15" t="n">
-        <v>1.266288114379083</v>
+        <v>1.2663</v>
       </c>
       <c r="G15" t="n">
         <v>0.2054099506572642</v>
@@ -2751,19 +2751,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.02730608243144142</v>
+        <v>0.0273</v>
       </c>
       <c r="C16" t="n">
-        <v>0.008604047380252196</v>
+        <v>0.0086</v>
       </c>
       <c r="D16" t="n">
-        <v>0.02447944447961795</v>
+        <v>0.0245</v>
       </c>
       <c r="E16" t="n">
-        <v>0.007713384029866039</v>
+        <v>0.0077</v>
       </c>
       <c r="F16" t="n">
-        <v>3.173632271495121</v>
+        <v>3.1736</v>
       </c>
       <c r="G16" t="n">
         <v>0.001505442893215186</v>
@@ -2776,19 +2776,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.08791933960749647</v>
+        <v>0.08790000000000001</v>
       </c>
       <c r="C17" t="n">
-        <v>0.01732298898188624</v>
+        <v>0.0173</v>
       </c>
       <c r="D17" t="n">
-        <v>0.05954487786088768</v>
+        <v>0.0595</v>
       </c>
       <c r="E17" t="n">
-        <v>0.01173229084427709</v>
+        <v>0.0117</v>
       </c>
       <c r="F17" t="n">
-        <v>5.075298477614296</v>
+        <v>5.0753</v>
       </c>
       <c r="G17" t="n">
         <v>3.868882024923099e-07</v>
@@ -2801,19 +2801,19 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.0542443387540471</v>
+        <v>0.0542</v>
       </c>
       <c r="C18" t="n">
-        <v>0.02308261176152301</v>
+        <v>0.0231</v>
       </c>
       <c r="D18" t="n">
-        <v>0.02288343080118621</v>
+        <v>0.0229</v>
       </c>
       <c r="E18" t="n">
-        <v>0.009737594025257607</v>
+        <v>0.0097</v>
       </c>
       <c r="F18" t="n">
-        <v>2.350008712812488</v>
+        <v>2.35</v>
       </c>
       <c r="G18" t="n">
         <v>0.01877297163093312</v>
@@ -2826,19 +2826,19 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.04678883689359144</v>
+        <v>0.0468</v>
       </c>
       <c r="C19" t="n">
-        <v>0.0234889149538298</v>
+        <v>0.0235</v>
       </c>
       <c r="D19" t="n">
-        <v>0.01398388554548594</v>
+        <v>0.014</v>
       </c>
       <c r="E19" t="n">
-        <v>0.007020185157605366</v>
+        <v>0.007</v>
       </c>
       <c r="F19" t="n">
-        <v>1.991953948726893</v>
+        <v>1.992</v>
       </c>
       <c r="G19" t="n">
         <v>0.046376110863128</v>
@@ -2851,19 +2851,19 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-0.1021619368057968</v>
+        <v>-0.1022</v>
       </c>
       <c r="C20" t="n">
-        <v>0.004974944117678012</v>
+        <v>0.005</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.1996522773328006</v>
+        <v>-0.1997</v>
       </c>
       <c r="E20" t="n">
-        <v>0.009722397144701314</v>
+        <v>0.0097</v>
       </c>
       <c r="F20" t="n">
-        <v>-20.53529333983344</v>
+        <v>-20.5353</v>
       </c>
       <c r="G20" t="n">
         <v>1.041834936009393e-93</v>
@@ -2876,19 +2876,19 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-0.1019076787667108</v>
+        <v>-0.1019</v>
       </c>
       <c r="C21" t="n">
-        <v>0.005449899312128422</v>
+        <v>0.0054</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.1739300660131559</v>
+        <v>-0.1739</v>
       </c>
       <c r="E21" t="n">
-        <v>0.00930156940669314</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="F21" t="n">
-        <v>-18.69900211549255</v>
+        <v>-18.699</v>
       </c>
       <c r="G21" t="n">
         <v>5.043982096799466e-78</v>
@@ -2901,19 +2901,19 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>-0.1214543165837861</v>
+        <v>-0.1215</v>
       </c>
       <c r="C22" t="n">
-        <v>0.007254663836294343</v>
+        <v>0.0073</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.1595870900986786</v>
+        <v>-0.1596</v>
       </c>
       <c r="E22" t="n">
-        <v>0.00953239640914408</v>
+        <v>0.0095</v>
       </c>
       <c r="F22" t="n">
-        <v>-16.74154989458816</v>
+        <v>-16.7415</v>
       </c>
       <c r="G22" t="n">
         <v>6.526643723517673e-63</v>
@@ -2926,19 +2926,19 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-0.07031173417326558</v>
+        <v>-0.0703</v>
       </c>
       <c r="C23" t="n">
-        <v>0.005972164892425402</v>
+        <v>0.006</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.137291866324466</v>
+        <v>-0.1373</v>
       </c>
       <c r="E23" t="n">
-        <v>0.01166134890170718</v>
+        <v>0.0117</v>
       </c>
       <c r="F23" t="n">
-        <v>-11.77324059863838</v>
+        <v>-11.7732</v>
       </c>
       <c r="G23" t="n">
         <v>5.362426103971977e-32</v>
@@ -2951,19 +2951,19 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>-0.1013615948052559</v>
+        <v>-0.1014</v>
       </c>
       <c r="C24" t="n">
-        <v>0.007673153890562856</v>
+        <v>0.0077</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.1150911202181795</v>
+        <v>-0.1151</v>
       </c>
       <c r="E24" t="n">
-        <v>0.00871248995803655</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="F24" t="n">
-        <v>-13.20989989916918</v>
+        <v>-13.2099</v>
       </c>
       <c r="G24" t="n">
         <v>7.692666028543185e-40</v>
@@ -3027,15 +3027,15 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.09876958677948304</v>
+        <v>0.0988</v>
       </c>
       <c r="C2" t="n">
-        <v>0.003476687483970993</v>
+        <v>0.0035</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>28.40910701202015</v>
+        <v>28.4091</v>
       </c>
       <c r="G2" t="n">
         <v>1.56071571869917e-177</v>
@@ -3048,19 +3048,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.02585194293462881</v>
+        <v>0.0259</v>
       </c>
       <c r="C3" t="n">
-        <v>0.001625507782373451</v>
+        <v>0.0016</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2115450765187038</v>
+        <v>0.2115</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01330144388270822</v>
+        <v>0.0133</v>
       </c>
       <c r="F3" t="n">
-        <v>15.90391828015836</v>
+        <v>15.9039</v>
       </c>
       <c r="G3" t="n">
         <v>5.952253279975866e-57</v>
@@ -3073,19 +3073,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.05370715533004308</v>
+        <v>-0.0537</v>
       </c>
       <c r="C4" t="n">
-        <v>0.002410693064033643</v>
+        <v>0.0024</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.2596277166110388</v>
+        <v>-0.2596</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01165361918386716</v>
+        <v>0.0117</v>
       </c>
       <c r="F4" t="n">
-        <v>-22.27871981353722</v>
+        <v>-22.2787</v>
       </c>
       <c r="G4" t="n">
         <v>5.943237171671356e-110</v>
@@ -3098,19 +3098,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.001789982428150638</v>
+        <v>0.0018</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0001721155220829719</v>
+        <v>0.0002</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0909008169992838</v>
+        <v>0.09089999999999999</v>
       </c>
       <c r="E5" t="n">
-        <v>0.008740555957169296</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>10.39988960024035</v>
+        <v>10.3999</v>
       </c>
       <c r="G5" t="n">
         <v>2.482206125847451e-25</v>
@@ -3123,19 +3123,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.02664330489333342</v>
+        <v>0.0266</v>
       </c>
       <c r="C6" t="n">
-        <v>0.003269903538677247</v>
+        <v>0.0033</v>
       </c>
       <c r="D6" t="n">
-        <v>0.104789915597705</v>
+        <v>0.1048</v>
       </c>
       <c r="E6" t="n">
-        <v>0.01286075121695442</v>
+        <v>0.0129</v>
       </c>
       <c r="F6" t="n">
-        <v>8.148040019587629</v>
+        <v>8.148</v>
       </c>
       <c r="G6" t="n">
         <v>3.698699617754467e-16</v>
@@ -3148,19 +3148,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.03331063289804159</v>
+        <v>0.0333</v>
       </c>
       <c r="C7" t="n">
-        <v>0.003469981940692815</v>
+        <v>0.0035</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1277329348017079</v>
+        <v>0.1277</v>
       </c>
       <c r="E7" t="n">
-        <v>0.01330599086334616</v>
+        <v>0.0133</v>
       </c>
       <c r="F7" t="n">
-        <v>9.599655983048372</v>
+        <v>9.5997</v>
       </c>
       <c r="G7" t="n">
         <v>8.021169245052314e-22</v>
@@ -3173,19 +3173,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.03253244482086735</v>
+        <v>0.0325</v>
       </c>
       <c r="C8" t="n">
-        <v>0.003312157832152412</v>
+        <v>0.0033</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1045299611148927</v>
+        <v>0.1045</v>
       </c>
       <c r="E8" t="n">
-        <v>0.01064229052896763</v>
+        <v>0.0106</v>
       </c>
       <c r="F8" t="n">
-        <v>9.82213000390929</v>
+        <v>9.822100000000001</v>
       </c>
       <c r="G8" t="n">
         <v>9.041266072722864e-23</v>
@@ -3198,19 +3198,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.02017408230158348</v>
+        <v>0.0202</v>
       </c>
       <c r="C9" t="n">
-        <v>0.00301505432183787</v>
+        <v>0.003</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0553096975563893</v>
+        <v>0.0553</v>
       </c>
       <c r="E9" t="n">
-        <v>0.008266137718881407</v>
+        <v>0.0083</v>
       </c>
       <c r="F9" t="n">
-        <v>6.691117355818013</v>
+        <v>6.6911</v>
       </c>
       <c r="G9" t="n">
         <v>2.214729568316151e-11</v>
@@ -3223,19 +3223,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.04667305348598745</v>
+        <v>0.0467</v>
       </c>
       <c r="C10" t="n">
-        <v>0.00469720135923217</v>
+        <v>0.0047</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1434937441943221</v>
+        <v>0.1435</v>
       </c>
       <c r="E10" t="n">
-        <v>0.01444128806514111</v>
+        <v>0.0144</v>
       </c>
       <c r="F10" t="n">
-        <v>9.936353568120589</v>
+        <v>9.936400000000001</v>
       </c>
       <c r="G10" t="n">
         <v>2.892208930517625e-23</v>
@@ -3248,19 +3248,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0212175155257281</v>
+        <v>0.0212</v>
       </c>
       <c r="C11" t="n">
-        <v>0.00326493854102702</v>
+        <v>0.0033</v>
       </c>
       <c r="D11" t="n">
-        <v>0.06528278255837758</v>
+        <v>0.0653</v>
       </c>
       <c r="E11" t="n">
-        <v>0.01004567535637607</v>
+        <v>0.01</v>
       </c>
       <c r="F11" t="n">
-        <v>6.498595688436424</v>
+        <v>6.4986</v>
       </c>
       <c r="G11" t="n">
         <v>8.107322170513796e-11</v>
@@ -3273,19 +3273,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.02762940447276075</v>
+        <v>0.0276</v>
       </c>
       <c r="C12" t="n">
-        <v>0.003235631339237121</v>
+        <v>0.0032</v>
       </c>
       <c r="D12" t="n">
-        <v>0.07010716030727027</v>
+        <v>0.0701</v>
       </c>
       <c r="E12" t="n">
-        <v>0.008210127193250297</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="F12" t="n">
-        <v>8.539107696760984</v>
+        <v>8.539099999999999</v>
       </c>
       <c r="G12" t="n">
         <v>1.352622650770721e-17</v>
@@ -3298,19 +3298,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.02057661116401539</v>
+        <v>0.0206</v>
       </c>
       <c r="C13" t="n">
-        <v>0.003456560515180043</v>
+        <v>0.0035</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0522113235874552</v>
+        <v>0.0522</v>
       </c>
       <c r="E13" t="n">
-        <v>0.00877071535828489</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="F13" t="n">
-        <v>5.952915065033545</v>
+        <v>5.9529</v>
       </c>
       <c r="G13" t="n">
         <v>2.63408016266086e-09</v>
@@ -3323,19 +3323,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.01711383370618993</v>
+        <v>0.0171</v>
       </c>
       <c r="C14" t="n">
-        <v>0.003833596306944397</v>
+        <v>0.0038</v>
       </c>
       <c r="D14" t="n">
-        <v>0.03616788187595865</v>
+        <v>0.0362</v>
       </c>
       <c r="E14" t="n">
-        <v>0.008101811713849166</v>
+        <v>0.0081</v>
       </c>
       <c r="F14" t="n">
-        <v>4.464172107842693</v>
+        <v>4.4642</v>
       </c>
       <c r="G14" t="n">
         <v>8.037893656124215e-06</v>
@@ -3348,19 +3348,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.004852455773411404</v>
+        <v>0.0049</v>
       </c>
       <c r="C15" t="n">
-        <v>0.003026204169000148</v>
+        <v>0.003</v>
       </c>
       <c r="D15" t="n">
-        <v>0.00953347009579103</v>
+        <v>0.0095</v>
       </c>
       <c r="E15" t="n">
-        <v>0.005945489932541639</v>
+        <v>0.0059</v>
       </c>
       <c r="F15" t="n">
-        <v>1.603479310192956</v>
+        <v>1.6035</v>
       </c>
       <c r="G15" t="n">
         <v>0.1088288734084694</v>
@@ -3373,19 +3373,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.01487801260484227</v>
+        <v>0.0149</v>
       </c>
       <c r="C16" t="n">
-        <v>0.002894534065671969</v>
+        <v>0.0029</v>
       </c>
       <c r="D16" t="n">
-        <v>0.03073597936671928</v>
+        <v>0.0307</v>
       </c>
       <c r="E16" t="n">
-        <v>0.005979719313438698</v>
+        <v>0.006</v>
       </c>
       <c r="F16" t="n">
-        <v>5.140037141483192</v>
+        <v>5.14</v>
       </c>
       <c r="G16" t="n">
         <v>2.746841668685638e-07</v>
@@ -3398,19 +3398,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.02977754030146236</v>
+        <v>0.0298</v>
       </c>
       <c r="C17" t="n">
-        <v>0.007507123208594828</v>
+        <v>0.0075</v>
       </c>
       <c r="D17" t="n">
-        <v>0.04323348094376889</v>
+        <v>0.0432</v>
       </c>
       <c r="E17" t="n">
-        <v>0.01089945861530312</v>
+        <v>0.0109</v>
       </c>
       <c r="F17" t="n">
-        <v>3.966571411452307</v>
+        <v>3.9666</v>
       </c>
       <c r="G17" t="n">
         <v>7.291393614817315e-05</v>
@@ -3423,19 +3423,19 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.01645443665330604</v>
+        <v>0.0165</v>
       </c>
       <c r="C18" t="n">
-        <v>0.007074380159691944</v>
+        <v>0.0071</v>
       </c>
       <c r="D18" t="n">
-        <v>0.01584433639750718</v>
+        <v>0.0158</v>
       </c>
       <c r="E18" t="n">
-        <v>0.006812075151262545</v>
+        <v>0.0068</v>
       </c>
       <c r="F18" t="n">
-        <v>2.325919201665091</v>
+        <v>2.3259</v>
       </c>
       <c r="G18" t="n">
         <v>0.02002286147083859</v>
@@ -3448,19 +3448,19 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.00907438193967503</v>
+        <v>0.0091</v>
       </c>
       <c r="C19" t="n">
-        <v>0.007403063502005415</v>
+        <v>0.0074</v>
       </c>
       <c r="D19" t="n">
-        <v>0.006308837114027716</v>
+        <v>0.0063</v>
       </c>
       <c r="E19" t="n">
-        <v>0.005146876348101823</v>
+        <v>0.0051</v>
       </c>
       <c r="F19" t="n">
-        <v>1.225760381120177</v>
+        <v>1.2258</v>
       </c>
       <c r="G19" t="n">
         <v>0.2202888603984025</v>
@@ -3473,19 +3473,19 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-0.05994786740940758</v>
+        <v>-0.0599</v>
       </c>
       <c r="C20" t="n">
-        <v>0.00211407167779509</v>
+        <v>0.0021</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.2679187499639367</v>
+        <v>-0.2679</v>
       </c>
       <c r="E20" t="n">
-        <v>0.009448200006529977</v>
+        <v>0.0094</v>
       </c>
       <c r="F20" t="n">
-        <v>-28.35659170834326</v>
+        <v>-28.3566</v>
       </c>
       <c r="G20" t="n">
         <v>6.941543432780558e-177</v>
@@ -3498,19 +3498,19 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-0.05870536656163572</v>
+        <v>-0.0587</v>
       </c>
       <c r="C21" t="n">
-        <v>0.00232773186094211</v>
+        <v>0.0023</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.2236168427444969</v>
+        <v>-0.2236</v>
       </c>
       <c r="E21" t="n">
-        <v>0.008866651892091407</v>
+        <v>0.0089</v>
       </c>
       <c r="F21" t="n">
-        <v>-25.21998669463403</v>
+        <v>-25.22</v>
       </c>
       <c r="G21" t="n">
         <v>2.418274690132437e-140</v>
@@ -3523,19 +3523,19 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>-0.07250601745455511</v>
+        <v>-0.0725</v>
       </c>
       <c r="C22" t="n">
-        <v>0.002746691218474138</v>
+        <v>0.0027</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.1979657342389056</v>
+        <v>-0.198</v>
       </c>
       <c r="E22" t="n">
-        <v>0.007499387814723046</v>
+        <v>0.0075</v>
       </c>
       <c r="F22" t="n">
-        <v>-26.39758592698097</v>
+        <v>-26.3976</v>
       </c>
       <c r="G22" t="n">
         <v>1.460463677895199e-153</v>
@@ -3548,19 +3548,19 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-0.04802488663967763</v>
+        <v>-0.048</v>
       </c>
       <c r="C23" t="n">
-        <v>0.002631729676753548</v>
+        <v>0.0026</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.2042551850982722</v>
+        <v>-0.2043</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0111930390650792</v>
+        <v>0.0112</v>
       </c>
       <c r="F23" t="n">
-        <v>-18.24841170576464</v>
+        <v>-18.2484</v>
       </c>
       <c r="G23" t="n">
         <v>2.130127519517401e-74</v>
@@ -3573,19 +3573,19 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>-0.03568878765466108</v>
+        <v>-0.0357</v>
       </c>
       <c r="C24" t="n">
-        <v>0.003754901798871801</v>
+        <v>0.0038</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.09209760362802473</v>
+        <v>-0.0921</v>
       </c>
       <c r="E24" t="n">
-        <v>0.00968980680657801</v>
+        <v>0.0097</v>
       </c>
       <c r="F24" t="n">
-        <v>-9.504586155990589</v>
+        <v>-9.5046</v>
       </c>
       <c r="G24" t="n">
         <v>2.008450123393033e-21</v>

</xml_diff>

<commit_message>
change in coef and vif by model update 1.1
</commit_message>
<xml_diff>
--- a/output/coefficients/standardized/standardized_ALL.xlsx
+++ b/output/coefficients/standardized/standardized_ALL.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,7 +464,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.4783</v>
+        <v>0.5096000000000001</v>
       </c>
       <c r="C2" t="n">
         <v>0.0103</v>
@@ -472,7 +472,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>46.4039</v>
+        <v>49.3949</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -485,22 +485,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1115</v>
+        <v>0.1076</v>
       </c>
       <c r="C3" t="n">
         <v>0.0049</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2412</v>
+        <v>0.2328</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0107</v>
+        <v>0.0106</v>
       </c>
       <c r="F3" t="n">
-        <v>22.6105</v>
+        <v>21.9733</v>
       </c>
       <c r="G3" t="n">
-        <v>3.416844086692463e-113</v>
+        <v>5.19024484586208e-107</v>
       </c>
     </row>
     <row r="4">
@@ -510,22 +510,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.2647</v>
+        <v>-0.2455</v>
       </c>
       <c r="C4" t="n">
         <v>0.0075</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.3504</v>
+        <v>-0.3251</v>
       </c>
       <c r="E4" t="n">
         <v>0.009900000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>-35.3137</v>
+        <v>-32.7927</v>
       </c>
       <c r="G4" t="n">
-        <v>3.613434805884537e-273</v>
+        <v>7.492269383312129e-236</v>
       </c>
     </row>
     <row r="5">
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.0012</v>
+        <v>-0.0015</v>
       </c>
       <c r="C5" t="n">
         <v>0.0005</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.0177</v>
+        <v>-0.022</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0081</v>
+        <v>0.007900000000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>-2.1892</v>
+        <v>-2.768</v>
       </c>
       <c r="G5" t="n">
-        <v>0.02858197558367184</v>
+        <v>0.005640304136887425</v>
       </c>
     </row>
     <row r="6">
@@ -560,22 +560,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.0663</v>
+        <v>0.0529</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0092</v>
+        <v>0.0091</v>
       </c>
       <c r="D6" t="n">
-        <v>0.07530000000000001</v>
+        <v>0.0601</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0104</v>
+        <v>0.0103</v>
       </c>
       <c r="F6" t="n">
-        <v>7.222</v>
+        <v>5.8113</v>
       </c>
       <c r="G6" t="n">
-        <v>5.121491758353771e-13</v>
+        <v>6.199053613937379e-09</v>
       </c>
     </row>
     <row r="7">
@@ -585,22 +585,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.09660000000000001</v>
+        <v>0.0706</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0098</v>
+        <v>0.0097</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1037</v>
+        <v>0.07580000000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0105</v>
+        <v>0.0104</v>
       </c>
       <c r="F7" t="n">
-        <v>9.8452</v>
+        <v>7.2972</v>
       </c>
       <c r="G7" t="n">
-        <v>7.18864398705146e-23</v>
+        <v>2.937960448986889e-13</v>
       </c>
     </row>
     <row r="8">
@@ -610,22 +610,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.0625</v>
+        <v>0.0592</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0092</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0607</v>
+        <v>0.0574</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0089</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="F8" t="n">
-        <v>6.8139</v>
+        <v>6.5405</v>
       </c>
       <c r="G8" t="n">
-        <v>9.501335183611905e-12</v>
+        <v>6.129438846606865e-11</v>
       </c>
     </row>
     <row r="9">
@@ -635,22 +635,22 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.0034</v>
+        <v>0.009900000000000001</v>
       </c>
       <c r="C9" t="n">
-        <v>0.008399999999999999</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.0032</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0078</v>
+        <v>0.0077</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.4046</v>
+        <v>1.2043</v>
       </c>
       <c r="G9" t="n">
-        <v>0.6857492507426544</v>
+        <v>0.2284826860528429</v>
       </c>
     </row>
     <row r="10">
@@ -660,22 +660,22 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.14</v>
+        <v>0.1313</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0144</v>
+        <v>0.014</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1163</v>
+        <v>0.109</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0119</v>
+        <v>0.0116</v>
       </c>
       <c r="F10" t="n">
-        <v>9.7369</v>
+        <v>9.3592</v>
       </c>
       <c r="G10" t="n">
-        <v>2.099345818653748e-22</v>
+        <v>8.034314722850815e-21</v>
       </c>
     </row>
     <row r="11">
@@ -685,22 +685,22 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.044</v>
+        <v>0.0449</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0106</v>
+        <v>0.0104</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0361</v>
+        <v>0.0368</v>
       </c>
       <c r="E11" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>4.1643</v>
+        <v>4.3228</v>
       </c>
       <c r="G11" t="n">
-        <v>3.123713916089543e-05</v>
+        <v>1.54082537388473e-05</v>
       </c>
     </row>
     <row r="12">
@@ -710,22 +710,22 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.0736</v>
+        <v>0.06419999999999999</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0113</v>
+        <v>0.011</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0541</v>
+        <v>0.0473</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0083</v>
+        <v>0.0081</v>
       </c>
       <c r="F12" t="n">
-        <v>6.4922</v>
+        <v>5.8224</v>
       </c>
       <c r="G12" t="n">
-        <v>8.459867074906337e-11</v>
+        <v>5.801343260495562e-09</v>
       </c>
     </row>
     <row r="13">
@@ -735,22 +735,22 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.0556</v>
+        <v>0.0434</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0118</v>
+        <v>0.0116</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0379</v>
+        <v>0.0295</v>
       </c>
       <c r="E13" t="n">
-        <v>0.0081</v>
+        <v>0.007900000000000001</v>
       </c>
       <c r="F13" t="n">
-        <v>4.7019</v>
+        <v>3.7416</v>
       </c>
       <c r="G13" t="n">
-        <v>2.57792917769175e-06</v>
+        <v>0.0001828608945014619</v>
       </c>
     </row>
     <row r="14">
@@ -760,22 +760,22 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.0402</v>
+        <v>0.0347</v>
       </c>
       <c r="C14" t="n">
-        <v>0.0122</v>
+        <v>0.012</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0254</v>
+        <v>0.0219</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0077</v>
+        <v>0.0075</v>
       </c>
       <c r="F14" t="n">
-        <v>3.3113</v>
+        <v>2.9029</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0009285897517735443</v>
+        <v>0.003697766179605234</v>
       </c>
     </row>
     <row r="15">
@@ -785,22 +785,22 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.0302</v>
+        <v>-0.0391</v>
       </c>
       <c r="C15" t="n">
-        <v>0.01</v>
+        <v>0.0098</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.0179</v>
+        <v>-0.0231</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0059</v>
+        <v>0.0058</v>
       </c>
       <c r="F15" t="n">
-        <v>-3.0257</v>
+        <v>-3.9877</v>
       </c>
       <c r="G15" t="n">
-        <v>0.002480177768151905</v>
+        <v>6.671685620093757e-05</v>
       </c>
     </row>
     <row r="16">
@@ -810,22 +810,22 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.0015</v>
+        <v>0.0118</v>
       </c>
       <c r="C16" t="n">
-        <v>0.0105</v>
+        <v>0.0106</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.0009</v>
+        <v>0.0068</v>
       </c>
       <c r="E16" t="n">
         <v>0.006</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.1446</v>
+        <v>1.1205</v>
       </c>
       <c r="G16" t="n">
-        <v>0.8850184701674246</v>
+        <v>0.2625053442913986</v>
       </c>
     </row>
     <row r="17">
@@ -835,22 +835,22 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.115</v>
+        <v>0.0912</v>
       </c>
       <c r="C17" t="n">
-        <v>0.0236</v>
+        <v>0.0232</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0453</v>
+        <v>0.036</v>
       </c>
       <c r="E17" t="n">
-        <v>0.009299999999999999</v>
+        <v>0.0091</v>
       </c>
       <c r="F17" t="n">
-        <v>4.8718</v>
+        <v>3.9356</v>
       </c>
       <c r="G17" t="n">
-        <v>1.105636634491079e-06</v>
+        <v>8.297693984728184e-05</v>
       </c>
     </row>
     <row r="18">
@@ -860,22 +860,22 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-0.0626</v>
+        <v>-0.0266</v>
       </c>
       <c r="C18" t="n">
         <v>0.008800000000000001</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.0217</v>
+        <v>-0.0092</v>
       </c>
       <c r="E18" t="n">
         <v>0.0031</v>
       </c>
       <c r="F18" t="n">
-        <v>-7.0824</v>
+        <v>-3.016</v>
       </c>
       <c r="G18" t="n">
-        <v>1.416818879886341e-12</v>
+        <v>0.002561019149257387</v>
       </c>
     </row>
     <row r="19">
@@ -885,22 +885,22 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.0863</v>
+        <v>0.0602</v>
       </c>
       <c r="C19" t="n">
-        <v>0.0252</v>
+        <v>0.0246</v>
       </c>
       <c r="D19" t="n">
-        <v>0.025</v>
+        <v>0.0175</v>
       </c>
       <c r="E19" t="n">
-        <v>0.0073</v>
+        <v>0.0071</v>
       </c>
       <c r="F19" t="n">
-        <v>3.418</v>
+        <v>2.4446</v>
       </c>
       <c r="G19" t="n">
-        <v>0.0006307360247045329</v>
+        <v>0.01450079799139041</v>
       </c>
     </row>
     <row r="20">
@@ -910,22 +910,22 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.0565</v>
+        <v>0.0165</v>
       </c>
       <c r="C20" t="n">
-        <v>0.0308</v>
+        <v>0.0309</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0114</v>
+        <v>0.0033</v>
       </c>
       <c r="E20" t="n">
         <v>0.0062</v>
       </c>
       <c r="F20" t="n">
-        <v>1.8353</v>
+        <v>0.5346</v>
       </c>
       <c r="G20" t="n">
-        <v>0.06645409798580651</v>
+        <v>0.5928969351046378</v>
       </c>
     </row>
     <row r="21">
@@ -935,22 +935,22 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-0.3082</v>
+        <v>-0.3222</v>
       </c>
       <c r="C21" t="n">
-        <v>0.0425</v>
+        <v>0.043</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.0439</v>
+        <v>-0.0459</v>
       </c>
       <c r="E21" t="n">
-        <v>0.006</v>
+        <v>0.0061</v>
       </c>
       <c r="F21" t="n">
-        <v>-7.2589</v>
+        <v>-7.4914</v>
       </c>
       <c r="G21" t="n">
-        <v>3.903585811780023e-13</v>
+        <v>6.812353441902274e-14</v>
       </c>
     </row>
     <row r="22">
@@ -960,22 +960,22 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>-0.1311</v>
+        <v>-0.1202</v>
       </c>
       <c r="C22" t="n">
-        <v>0.006</v>
+        <v>0.0059</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.1743</v>
+        <v>-0.1597</v>
       </c>
       <c r="E22" t="n">
-        <v>0.008</v>
+        <v>0.0078</v>
       </c>
       <c r="F22" t="n">
-        <v>-21.7685</v>
+        <v>-20.4092</v>
       </c>
       <c r="G22" t="n">
-        <v>4.618387003790065e-105</v>
+        <v>1.385639557257553e-92</v>
       </c>
     </row>
     <row r="23">
@@ -985,22 +985,22 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-0.1108</v>
+        <v>-0.1018</v>
       </c>
       <c r="C23" t="n">
-        <v>0.0075</v>
+        <v>0.0074</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.1152</v>
+        <v>-0.1059</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0078</v>
+        <v>0.0076</v>
       </c>
       <c r="F23" t="n">
-        <v>-14.7951</v>
+        <v>-13.8522</v>
       </c>
       <c r="G23" t="n">
-        <v>1.575873980804803e-49</v>
+        <v>1.233771683303811e-43</v>
       </c>
     </row>
     <row r="24">
@@ -1010,22 +1010,22 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>-0.2373</v>
+        <v>-0.2341</v>
       </c>
       <c r="C24" t="n">
-        <v>0.0095</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.1723</v>
+        <v>-0.1699</v>
       </c>
       <c r="E24" t="n">
-        <v>0.0069</v>
+        <v>0.0068</v>
       </c>
       <c r="F24" t="n">
-        <v>-25.1014</v>
+        <v>-25.0389</v>
       </c>
       <c r="G24" t="n">
-        <v>4.799422352546218e-139</v>
+        <v>2.307580081083772e-138</v>
       </c>
     </row>
     <row r="25">
@@ -1035,22 +1035,22 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>-0.0432</v>
+        <v>-0.0467</v>
       </c>
       <c r="C25" t="n">
-        <v>0.0083</v>
+        <v>0.0081</v>
       </c>
       <c r="D25" t="n">
-        <v>-0.0499</v>
+        <v>-0.0539</v>
       </c>
       <c r="E25" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0094</v>
       </c>
       <c r="F25" t="n">
-        <v>-5.2267</v>
+        <v>-5.7408</v>
       </c>
       <c r="G25" t="n">
-        <v>1.725851529309045e-07</v>
+        <v>9.422985697115229e-09</v>
       </c>
     </row>
     <row r="26">
@@ -1060,22 +1060,97 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>-0.1596</v>
+        <v>-0.1491</v>
       </c>
       <c r="C26" t="n">
+        <v>0.0063</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-0.1507</v>
+      </c>
+      <c r="E26" t="n">
         <v>0.0064</v>
       </c>
-      <c r="D26" t="n">
-        <v>-0.1613</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0.0065</v>
-      </c>
       <c r="F26" t="n">
-        <v>-24.8173</v>
+        <v>-23.6238</v>
       </c>
       <c r="G26" t="n">
-        <v>5.839207849537465e-136</v>
+        <v>2.196787974340853e-123</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>d_aa</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>-0.08890000000000001</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.0052</v>
+      </c>
+      <c r="D27" t="n">
+        <v>-0.1091</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.0064</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-17.0953</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1.609484180381554e-65</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>d_indie</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>-0.065</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.0066</v>
+      </c>
+      <c r="D28" t="n">
+        <v>-0.0611</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.0062</v>
+      </c>
+      <c r="F28" t="n">
+        <v>-9.814500000000001</v>
+      </c>
+      <c r="G28" t="n">
+        <v>9.7508750172815e-23</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>d_unknown</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>-0.1334</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.0047</v>
+      </c>
+      <c r="D29" t="n">
+        <v>-0.1503</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.0053</v>
+      </c>
+      <c r="F29" t="n">
+        <v>-28.5691</v>
+      </c>
+      <c r="G29" t="n">
+        <v>1.627152312090757e-179</v>
       </c>
     </row>
   </sheetData>
@@ -1089,7 +1164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1136,18 +1211,18 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2778</v>
+        <v>0.2985</v>
       </c>
       <c r="C2" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.0091</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>30.7105</v>
+        <v>32.7004</v>
       </c>
       <c r="G2" t="n">
-        <v>4.121846448096214e-207</v>
+        <v>1.543351766214401e-234</v>
       </c>
     </row>
     <row r="3">
@@ -1157,22 +1232,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.0784</v>
+        <v>0.0756</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0039</v>
+        <v>0.0038</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2574</v>
+        <v>0.2483</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0127</v>
+        <v>0.0126</v>
       </c>
       <c r="F3" t="n">
-        <v>20.3358</v>
+        <v>19.645</v>
       </c>
       <c r="G3" t="n">
-        <v>6.203109040878432e-92</v>
+        <v>6.379495164655918e-86</v>
       </c>
     </row>
     <row r="4">
@@ -1182,22 +1257,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.1549</v>
+        <v>-0.1424</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0059</v>
+        <v>0.006</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.2965</v>
+        <v>-0.2726</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0113</v>
+        <v>0.0114</v>
       </c>
       <c r="F4" t="n">
-        <v>-26.1937</v>
+        <v>-23.8748</v>
       </c>
       <c r="G4" t="n">
-        <v>3.13217078813274e-151</v>
+        <v>5.600838401538451e-126</v>
       </c>
     </row>
     <row r="5">
@@ -1207,22 +1282,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.0013</v>
+        <v>-0.0017</v>
       </c>
       <c r="C5" t="n">
         <v>0.0005</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.026</v>
+        <v>-0.0341</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0092</v>
+        <v>0.0091</v>
       </c>
       <c r="F5" t="n">
-        <v>-2.8271</v>
+        <v>-3.7688</v>
       </c>
       <c r="G5" t="n">
-        <v>0.004696631178074946</v>
+        <v>0.0001640347282356813</v>
       </c>
     </row>
     <row r="6">
@@ -1232,22 +1307,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.0633</v>
+        <v>0.0548</v>
       </c>
       <c r="C6" t="n">
         <v>0.0092</v>
       </c>
       <c r="D6" t="n">
-        <v>0.09859999999999999</v>
+        <v>0.0852</v>
       </c>
       <c r="E6" t="n">
         <v>0.0144</v>
       </c>
       <c r="F6" t="n">
-        <v>6.851</v>
+        <v>5.9339</v>
       </c>
       <c r="G6" t="n">
-        <v>7.334199362201158e-12</v>
+        <v>2.957447492894423e-09</v>
       </c>
     </row>
     <row r="7">
@@ -1257,22 +1332,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.08069999999999999</v>
+        <v>0.0634</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0095</v>
+        <v>0.0094</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1208</v>
+        <v>0.0949</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0142</v>
+        <v>0.0141</v>
       </c>
       <c r="F7" t="n">
-        <v>8.521699999999999</v>
+        <v>6.7219</v>
       </c>
       <c r="G7" t="n">
-        <v>1.571753521963822e-17</v>
+        <v>1.79366847143131e-11</v>
       </c>
     </row>
     <row r="8">
@@ -1282,22 +1357,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.0772</v>
+        <v>0.0732</v>
       </c>
       <c r="C8" t="n">
         <v>0.0097</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0961</v>
+        <v>0.0911</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0121</v>
+        <v>0.012</v>
       </c>
       <c r="F8" t="n">
-        <v>7.9451</v>
+        <v>7.5619</v>
       </c>
       <c r="G8" t="n">
-        <v>1.940343772614067e-15</v>
+        <v>3.972147382998328e-14</v>
       </c>
     </row>
     <row r="9">
@@ -1307,22 +1382,22 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.0343</v>
+        <v>0.0348</v>
       </c>
       <c r="C9" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0095</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0358</v>
+        <v>0.0363</v>
       </c>
       <c r="E9" t="n">
-        <v>0.01</v>
+        <v>0.009900000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>3.5752</v>
+        <v>3.6551</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0003499062625434746</v>
+        <v>0.0002570401520009639</v>
       </c>
     </row>
     <row r="10">
@@ -1332,22 +1407,22 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.1112</v>
+        <v>0.1057</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0126</v>
+        <v>0.0124</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1357</v>
+        <v>0.129</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0154</v>
+        <v>0.0151</v>
       </c>
       <c r="F10" t="n">
-        <v>8.8146</v>
+        <v>8.5166</v>
       </c>
       <c r="G10" t="n">
-        <v>1.201387264815336e-18</v>
+        <v>1.643557135152196e-17</v>
       </c>
     </row>
     <row r="11">
@@ -1357,22 +1432,22 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0244</v>
+        <v>0.0255</v>
       </c>
       <c r="C11" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0095</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0294</v>
+        <v>0.0308</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0115</v>
+        <v>0.0114</v>
       </c>
       <c r="F11" t="n">
-        <v>2.5562</v>
+        <v>2.7004</v>
       </c>
       <c r="G11" t="n">
-        <v>0.01058239055606917</v>
+        <v>0.006924581632716168</v>
       </c>
     </row>
     <row r="12">
@@ -1382,22 +1457,22 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.0776</v>
+        <v>0.0697</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0111</v>
+        <v>0.0108</v>
       </c>
       <c r="D12" t="n">
-        <v>0.07480000000000001</v>
+        <v>0.0672</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0107</v>
+        <v>0.0104</v>
       </c>
       <c r="F12" t="n">
-        <v>7.0012</v>
+        <v>6.4358</v>
       </c>
       <c r="G12" t="n">
-        <v>2.537127339931194e-12</v>
+        <v>1.228204934607188e-10</v>
       </c>
     </row>
     <row r="13">
@@ -1407,22 +1482,22 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.0385</v>
+        <v>0.0309</v>
       </c>
       <c r="C13" t="n">
+        <v>0.009900000000000001</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.0314</v>
+      </c>
+      <c r="E13" t="n">
         <v>0.01</v>
       </c>
-      <c r="D13" t="n">
-        <v>0.039</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0.0102</v>
-      </c>
       <c r="F13" t="n">
-        <v>3.8432</v>
+        <v>3.1219</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0001214406303753483</v>
+        <v>0.001796715394070818</v>
       </c>
     </row>
     <row r="14">
@@ -1432,22 +1507,22 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.0561</v>
+        <v>0.0555</v>
       </c>
       <c r="C14" t="n">
-        <v>0.0118</v>
+        <v>0.0116</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0471</v>
+        <v>0.0466</v>
       </c>
       <c r="E14" t="n">
-        <v>0.009900000000000001</v>
+        <v>0.0098</v>
       </c>
       <c r="F14" t="n">
-        <v>4.7635</v>
+        <v>4.7745</v>
       </c>
       <c r="G14" t="n">
-        <v>1.902903654966833e-06</v>
+        <v>1.801970706125262e-06</v>
       </c>
     </row>
     <row r="15">
@@ -1457,22 +1532,22 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.0274</v>
+        <v>-0.0307</v>
       </c>
       <c r="C15" t="n">
-        <v>0.0106</v>
+        <v>0.0105</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.0187</v>
+        <v>-0.021</v>
       </c>
       <c r="E15" t="n">
         <v>0.0072</v>
       </c>
       <c r="F15" t="n">
-        <v>-2.5935</v>
+        <v>-2.9153</v>
       </c>
       <c r="G15" t="n">
-        <v>0.009499853553076362</v>
+        <v>0.003553300905034483</v>
       </c>
     </row>
     <row r="16">
@@ -1482,22 +1557,22 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.005</v>
+        <v>0.0171</v>
       </c>
       <c r="C16" t="n">
         <v>0.0102</v>
       </c>
       <c r="D16" t="n">
-        <v>0.0039</v>
+        <v>0.0134</v>
       </c>
       <c r="E16" t="n">
         <v>0.008</v>
       </c>
       <c r="F16" t="n">
-        <v>0.4918</v>
+        <v>1.6731</v>
       </c>
       <c r="G16" t="n">
-        <v>0.6228339559200247</v>
+        <v>0.09430899476652224</v>
       </c>
     </row>
     <row r="17">
@@ -1507,22 +1582,22 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.066</v>
+        <v>0.051</v>
       </c>
       <c r="C17" t="n">
-        <v>0.0187</v>
+        <v>0.0185</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0372</v>
+        <v>0.0288</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0105</v>
+        <v>0.0104</v>
       </c>
       <c r="F17" t="n">
-        <v>3.5312</v>
+        <v>2.7568</v>
       </c>
       <c r="G17" t="n">
-        <v>0.0004136892471294721</v>
+        <v>0.005836821367813983</v>
       </c>
     </row>
     <row r="18">
@@ -1532,22 +1607,22 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.0742</v>
+        <v>0.0553</v>
       </c>
       <c r="C18" t="n">
-        <v>0.0253</v>
+        <v>0.025</v>
       </c>
       <c r="D18" t="n">
-        <v>0.0277</v>
+        <v>0.0207</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0095</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="F18" t="n">
-        <v>2.9285</v>
+        <v>2.2126</v>
       </c>
       <c r="G18" t="n">
-        <v>0.003406194983078177</v>
+        <v>0.02692379429928699</v>
       </c>
     </row>
     <row r="19">
@@ -1557,22 +1632,22 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.0323</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="C19" t="n">
-        <v>0.0227</v>
+        <v>0.0228</v>
       </c>
       <c r="D19" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0024</v>
       </c>
       <c r="E19" t="n">
         <v>0.0062</v>
       </c>
       <c r="F19" t="n">
-        <v>1.4251</v>
+        <v>0.3923</v>
       </c>
       <c r="G19" t="n">
-        <v>0.1541241609055243</v>
+        <v>0.6948626568191176</v>
       </c>
     </row>
     <row r="20">
@@ -1582,22 +1657,22 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-0.0612</v>
+        <v>-0.0504</v>
       </c>
       <c r="C20" t="n">
-        <v>0.0052</v>
+        <v>0.0051</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.1074</v>
+        <v>-0.08840000000000001</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0091</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="F20" t="n">
-        <v>-11.8073</v>
+        <v>-9.8391</v>
       </c>
       <c r="G20" t="n">
-        <v>3.578989638699906e-32</v>
+        <v>7.639268626007967e-23</v>
       </c>
     </row>
     <row r="21">
@@ -1607,22 +1682,22 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-0.0435</v>
+        <v>-0.0358</v>
       </c>
       <c r="C21" t="n">
-        <v>0.006</v>
+        <v>0.0059</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.06560000000000001</v>
+        <v>-0.054</v>
       </c>
       <c r="E21" t="n">
-        <v>0.0091</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="F21" t="n">
-        <v>-7.2382</v>
+        <v>-6.0283</v>
       </c>
       <c r="G21" t="n">
-        <v>4.546002757444119e-13</v>
+        <v>1.657370377219674e-09</v>
       </c>
     </row>
     <row r="22">
@@ -1632,22 +1707,22 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>-0.1573</v>
+        <v>-0.1594</v>
       </c>
       <c r="C22" t="n">
-        <v>0.012</v>
+        <v>0.0119</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.1115</v>
+        <v>-0.113</v>
       </c>
       <c r="E22" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.008399999999999999</v>
       </c>
       <c r="F22" t="n">
-        <v>-13.1369</v>
+        <v>-13.3933</v>
       </c>
       <c r="G22" t="n">
-        <v>2.024629328319839e-39</v>
+        <v>6.61841632152771e-41</v>
       </c>
     </row>
     <row r="23">
@@ -1657,22 +1732,22 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.0089</v>
+        <v>0.0062</v>
       </c>
       <c r="C23" t="n">
-        <v>0.0067</v>
+        <v>0.0066</v>
       </c>
       <c r="D23" t="n">
-        <v>0.0151</v>
+        <v>0.0106</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0114</v>
+        <v>0.0113</v>
       </c>
       <c r="F23" t="n">
-        <v>1.3237</v>
+        <v>0.9374</v>
       </c>
       <c r="G23" t="n">
-        <v>0.1856030841934638</v>
+        <v>0.3485507775861378</v>
       </c>
     </row>
     <row r="24">
@@ -1682,22 +1757,97 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>-0.1039</v>
+        <v>-0.1041</v>
       </c>
       <c r="C24" t="n">
         <v>0.0065</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.1058</v>
+        <v>-0.1059</v>
       </c>
       <c r="E24" t="n">
         <v>0.0066</v>
       </c>
       <c r="F24" t="n">
-        <v>-15.9663</v>
+        <v>-16.0391</v>
       </c>
       <c r="G24" t="n">
-        <v>2.195617844741011e-57</v>
+        <v>6.812758172713022e-58</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>d_aa</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>-0.0598</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.0046</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-0.1001</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-13.0236</v>
+      </c>
+      <c r="G25" t="n">
+        <v>8.988103653279595e-39</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>d_indie</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>-0.0427</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.0059</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-0.0538</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="F26" t="n">
+        <v>-7.2129</v>
+      </c>
+      <c r="G26" t="n">
+        <v>5.477667856739737e-13</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>d_unknown</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>-0.0973</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="D27" t="n">
+        <v>-0.1273</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.0066</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-19.3015</v>
+      </c>
+      <c r="G27" t="n">
+        <v>5.21533632665722e-83</v>
       </c>
     </row>
   </sheetData>
@@ -1711,7 +1861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1758,18 +1908,18 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1269</v>
+        <v>0.1393</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0056</v>
+        <v>0.0058</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>22.7903</v>
+        <v>24.0928</v>
       </c>
       <c r="G2" t="n">
-        <v>5.719919393903775e-115</v>
+        <v>2.973277728886143e-128</v>
       </c>
     </row>
     <row r="3">
@@ -1779,22 +1929,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.0127</v>
+        <v>0.0116</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0026</v>
+        <v>0.0025</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0738</v>
+        <v>0.06759999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0149</v>
+        <v>0.0147</v>
       </c>
       <c r="F3" t="n">
-        <v>4.9405</v>
+        <v>4.6011</v>
       </c>
       <c r="G3" t="n">
-        <v>7.792589020641442e-07</v>
+        <v>4.201972236188619e-06</v>
       </c>
     </row>
     <row r="4">
@@ -1804,22 +1954,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.0178</v>
+        <v>-0.0134</v>
       </c>
       <c r="C4" t="n">
         <v>0.0037</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.07489999999999999</v>
+        <v>-0.0565</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0158</v>
+        <v>0.0156</v>
       </c>
       <c r="F4" t="n">
-        <v>-4.7546</v>
+        <v>-3.6109</v>
       </c>
       <c r="G4" t="n">
-        <v>1.988349022704924e-06</v>
+        <v>0.0003051525889843639</v>
       </c>
     </row>
     <row r="5">
@@ -1829,22 +1979,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.0044</v>
+        <v>-0.0043</v>
       </c>
       <c r="C5" t="n">
         <v>0.0004</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.2003</v>
+        <v>-0.1965</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0161</v>
+        <v>0.016</v>
       </c>
       <c r="F5" t="n">
-        <v>-12.4537</v>
+        <v>-12.2809</v>
       </c>
       <c r="G5" t="n">
-        <v>1.334427727785046e-35</v>
+        <v>1.147278220178956e-34</v>
       </c>
     </row>
     <row r="6">
@@ -1854,22 +2004,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-0.0207</v>
+        <v>-0.0276</v>
       </c>
       <c r="C6" t="n">
-        <v>0.005</v>
+        <v>0.0051</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.07480000000000001</v>
+        <v>-0.0999</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0182</v>
+        <v>0.0183</v>
       </c>
       <c r="F6" t="n">
-        <v>-4.1141</v>
+        <v>-5.4657</v>
       </c>
       <c r="G6" t="n">
-        <v>3.886357916280625e-05</v>
+        <v>4.610764476576635e-08</v>
       </c>
     </row>
     <row r="7">
@@ -1879,22 +2029,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.0014</v>
+        <v>-0.0145</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0068</v>
+        <v>0.007</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.0039</v>
+        <v>-0.0416</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0197</v>
+        <v>0.0202</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.1983</v>
+        <v>-2.0558</v>
       </c>
       <c r="G7" t="n">
-        <v>0.8427909080393092</v>
+        <v>0.03979982084358254</v>
       </c>
     </row>
     <row r="8">
@@ -1904,22 +2054,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-0.0278</v>
+        <v>-0.0277</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0059</v>
+        <v>0.0058</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.0828</v>
+        <v>-0.0824</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0175</v>
+        <v>0.0173</v>
       </c>
       <c r="F8" t="n">
-        <v>-4.7231</v>
+        <v>-4.7519</v>
       </c>
       <c r="G8" t="n">
-        <v>2.322951006754869e-06</v>
+        <v>2.015223998359697e-06</v>
       </c>
     </row>
     <row r="9">
@@ -1929,22 +2079,22 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.0566</v>
+        <v>-0.0495</v>
       </c>
       <c r="C9" t="n">
         <v>0.0044</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.1982</v>
+        <v>-0.1734</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0154</v>
+        <v>0.0153</v>
       </c>
       <c r="F9" t="n">
-        <v>-12.8561</v>
+        <v>-11.3685</v>
       </c>
       <c r="G9" t="n">
-        <v>7.949098793573911e-38</v>
+        <v>6.003318545909891e-30</v>
       </c>
     </row>
     <row r="10">
@@ -1954,22 +2104,22 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-0.0371</v>
+        <v>-0.0439</v>
       </c>
       <c r="C10" t="n">
         <v>0.006</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.0905</v>
+        <v>-0.107</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0146</v>
+        <v>0.0147</v>
       </c>
       <c r="F10" t="n">
-        <v>-6.1938</v>
+        <v>-7.2786</v>
       </c>
       <c r="G10" t="n">
-        <v>5.871625820920273e-10</v>
+        <v>3.37288044545696e-13</v>
       </c>
     </row>
     <row r="11">
@@ -1979,22 +2129,22 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-0.0679</v>
+        <v>-0.0709</v>
       </c>
       <c r="C11" t="n">
         <v>0.0061</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.1229</v>
+        <v>-0.1281</v>
       </c>
       <c r="E11" t="n">
         <v>0.011</v>
       </c>
       <c r="F11" t="n">
-        <v>-11.1725</v>
+        <v>-11.6207</v>
       </c>
       <c r="G11" t="n">
-        <v>5.556307084838132e-29</v>
+        <v>3.233128502358928e-31</v>
       </c>
     </row>
     <row r="12">
@@ -2004,22 +2154,22 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.0342</v>
+        <v>-0.0344</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0073</v>
+        <v>0.0072</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.0728</v>
+        <v>-0.0732</v>
       </c>
       <c r="E12" t="n">
         <v>0.0154</v>
       </c>
       <c r="F12" t="n">
-        <v>-4.715</v>
+        <v>-4.7625</v>
       </c>
       <c r="G12" t="n">
-        <v>2.417144481668843e-06</v>
+        <v>1.91211945963566e-06</v>
       </c>
     </row>
     <row r="13">
@@ -2029,22 +2179,22 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-0.0336</v>
+        <v>-0.0439</v>
       </c>
       <c r="C13" t="n">
         <v>0.0091</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.0539</v>
+        <v>-0.0704</v>
       </c>
       <c r="E13" t="n">
         <v>0.0146</v>
       </c>
       <c r="F13" t="n">
-        <v>-3.6891</v>
+        <v>-4.8254</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0002250604045411201</v>
+        <v>1.397440453692042e-06</v>
       </c>
     </row>
     <row r="14">
@@ -2054,22 +2204,22 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.0282</v>
+        <v>-0.0294</v>
       </c>
       <c r="C14" t="n">
-        <v>0.0061</v>
+        <v>0.006</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.068</v>
+        <v>-0.0711</v>
       </c>
       <c r="E14" t="n">
         <v>0.0146</v>
       </c>
       <c r="F14" t="n">
-        <v>-4.6432</v>
+        <v>-4.8768</v>
       </c>
       <c r="G14" t="n">
-        <v>3.429742796471264e-06</v>
+        <v>1.078040353427481e-06</v>
       </c>
     </row>
     <row r="15">
@@ -2079,22 +2229,22 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.009299999999999999</v>
+        <v>-0.0156</v>
       </c>
       <c r="C15" t="n">
-        <v>0.008399999999999999</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.0177</v>
+        <v>-0.0295</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0159</v>
+        <v>0.0161</v>
       </c>
       <c r="F15" t="n">
-        <v>-1.1158</v>
+        <v>-1.8283</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2644871290746181</v>
+        <v>0.06750116419621574</v>
       </c>
     </row>
     <row r="16">
@@ -2104,22 +2254,22 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.034</v>
+        <v>-0.0412</v>
       </c>
       <c r="C16" t="n">
         <v>0.0086</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.0477</v>
+        <v>-0.0577</v>
       </c>
       <c r="E16" t="n">
         <v>0.012</v>
       </c>
       <c r="F16" t="n">
-        <v>-3.9727</v>
+        <v>-4.7911</v>
       </c>
       <c r="G16" t="n">
-        <v>7.105818977226174e-05</v>
+        <v>1.658427009483529e-06</v>
       </c>
     </row>
     <row r="17">
@@ -2129,22 +2279,22 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-0.0315</v>
+        <v>-0.042</v>
       </c>
       <c r="C17" t="n">
-        <v>0.0069</v>
+        <v>0.007</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.0401</v>
+        <v>-0.0535</v>
       </c>
       <c r="E17" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0089</v>
       </c>
       <c r="F17" t="n">
-        <v>-4.5574</v>
+        <v>-6.0261</v>
       </c>
       <c r="G17" t="n">
-        <v>5.178697854291059e-06</v>
+        <v>1.679855939870908e-09</v>
       </c>
     </row>
     <row r="18">
@@ -2154,22 +2304,22 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-0.049</v>
+        <v>-0.0375</v>
       </c>
       <c r="C18" t="n">
         <v>0.0044</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.0888</v>
+        <v>-0.068</v>
       </c>
       <c r="E18" t="n">
         <v>0.008</v>
       </c>
       <c r="F18" t="n">
-        <v>-11.1412</v>
+        <v>-8.5556</v>
       </c>
       <c r="G18" t="n">
-        <v>7.906114396722562e-29</v>
+        <v>1.172793169560562e-17</v>
       </c>
     </row>
     <row r="19">
@@ -2179,22 +2329,22 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.0244</v>
+        <v>0.0181</v>
       </c>
       <c r="C19" t="n">
-        <v>0.0166</v>
+        <v>0.0161</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0229</v>
+        <v>0.0169</v>
       </c>
       <c r="E19" t="n">
-        <v>0.0155</v>
+        <v>0.0151</v>
       </c>
       <c r="F19" t="n">
-        <v>1.4746</v>
+        <v>1.1194</v>
       </c>
       <c r="G19" t="n">
-        <v>0.1403202084202728</v>
+        <v>0.2629609945769958</v>
       </c>
     </row>
     <row r="20">
@@ -2204,22 +2354,22 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.029</v>
+        <v>0.0158</v>
       </c>
       <c r="C20" t="n">
-        <v>0.0235</v>
+        <v>0.0245</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0193</v>
+        <v>0.0105</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0156</v>
+        <v>0.0163</v>
       </c>
       <c r="F20" t="n">
-        <v>1.234</v>
+        <v>0.6433</v>
       </c>
       <c r="G20" t="n">
-        <v>0.2171959761181209</v>
+        <v>0.5200393055702741</v>
       </c>
     </row>
     <row r="21">
@@ -2229,22 +2379,22 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-0.0041</v>
+        <v>-0.0086</v>
       </c>
       <c r="C21" t="n">
-        <v>0.0166</v>
+        <v>0.0162</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.003</v>
+        <v>-0.0065</v>
       </c>
       <c r="E21" t="n">
-        <v>0.0124</v>
+        <v>0.0121</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.2449</v>
+        <v>-0.5315</v>
       </c>
       <c r="G21" t="n">
-        <v>0.806509111750946</v>
+        <v>0.5950808586216669</v>
       </c>
     </row>
     <row r="22">
@@ -2257,19 +2407,19 @@
         <v>0.0023</v>
       </c>
       <c r="C22" t="n">
-        <v>0.0038</v>
+        <v>0.0037</v>
       </c>
       <c r="D22" t="n">
         <v>0.009900000000000001</v>
       </c>
       <c r="E22" t="n">
-        <v>0.0162</v>
+        <v>0.016</v>
       </c>
       <c r="F22" t="n">
-        <v>0.6104000000000001</v>
+        <v>0.6157</v>
       </c>
       <c r="G22" t="n">
-        <v>0.5416244107718886</v>
+        <v>0.5381087955485305</v>
       </c>
     </row>
     <row r="23">
@@ -2279,22 +2429,22 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-0.0242</v>
+        <v>-0.0266</v>
       </c>
       <c r="C23" t="n">
         <v>0.0053</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.0589</v>
+        <v>-0.065</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0129</v>
+        <v>0.013</v>
       </c>
       <c r="F23" t="n">
-        <v>-4.5519</v>
+        <v>-4.9926</v>
       </c>
       <c r="G23" t="n">
-        <v>5.316557525235557e-06</v>
+        <v>5.955884042550342e-07</v>
       </c>
     </row>
     <row r="24">
@@ -2304,22 +2454,22 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>-0.0713</v>
+        <v>-0.07190000000000001</v>
       </c>
       <c r="C24" t="n">
         <v>0.0034</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.2003</v>
+        <v>-0.2017</v>
       </c>
       <c r="E24" t="n">
         <v>0.009599999999999999</v>
       </c>
       <c r="F24" t="n">
-        <v>-20.9511</v>
+        <v>-20.9874</v>
       </c>
       <c r="G24" t="n">
-        <v>1.833481854511251e-97</v>
+        <v>8.549389740776044e-98</v>
       </c>
     </row>
     <row r="25">
@@ -2329,22 +2479,97 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>-0.0178</v>
+        <v>-0.013</v>
       </c>
       <c r="C25" t="n">
-        <v>0.003</v>
+        <v>0.0029</v>
       </c>
       <c r="D25" t="n">
-        <v>-0.07630000000000001</v>
+        <v>-0.0557</v>
       </c>
       <c r="E25" t="n">
-        <v>0.0127</v>
+        <v>0.0125</v>
       </c>
       <c r="F25" t="n">
-        <v>-5.9922</v>
+        <v>-4.4549</v>
       </c>
       <c r="G25" t="n">
-        <v>2.069937966897287e-09</v>
+        <v>8.392923020292335e-06</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>d_aa</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>-0.0306</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.0033</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-0.1157</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.0124</v>
+      </c>
+      <c r="F26" t="n">
+        <v>-9.331</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1.048921794262594e-20</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>d_indie</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>-0.0367</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.0038</v>
+      </c>
+      <c r="D27" t="n">
+        <v>-0.0926</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.0095</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-9.7531</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1.78922769219574e-22</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>d_unknown</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>-0.0375</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.0033</v>
+      </c>
+      <c r="D28" t="n">
+        <v>-0.141</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.0123</v>
+      </c>
+      <c r="F28" t="n">
+        <v>-11.4551</v>
+      </c>
+      <c r="G28" t="n">
+        <v>2.21591782514193e-30</v>
       </c>
     </row>
   </sheetData>
@@ -2358,7 +2583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2405,7 +2630,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2223</v>
+        <v>0.2365</v>
       </c>
       <c r="C2" t="n">
         <v>0.008</v>
@@ -2413,10 +2638,10 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>27.9486</v>
+        <v>29.5134</v>
       </c>
       <c r="G2" t="n">
-        <v>6.848253084229291e-172</v>
+        <v>1.935312902244293e-191</v>
       </c>
     </row>
     <row r="3">
@@ -2426,22 +2651,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.0579</v>
+        <v>0.0561</v>
       </c>
       <c r="C3" t="n">
         <v>0.0033</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2255</v>
+        <v>0.2184</v>
       </c>
       <c r="E3" t="n">
         <v>0.0129</v>
       </c>
       <c r="F3" t="n">
-        <v>17.4134</v>
+        <v>16.9424</v>
       </c>
       <c r="G3" t="n">
-        <v>6.52548235122811e-68</v>
+        <v>2.188213823860349e-64</v>
       </c>
     </row>
     <row r="4">
@@ -2451,22 +2676,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.1165</v>
+        <v>-0.1091</v>
       </c>
       <c r="C4" t="n">
         <v>0.0053</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.2631</v>
+        <v>-0.2465</v>
       </c>
       <c r="E4" t="n">
         <v>0.0119</v>
       </c>
       <c r="F4" t="n">
-        <v>-22.1447</v>
+        <v>-20.7673</v>
       </c>
       <c r="G4" t="n">
-        <v>1.174196130163128e-108</v>
+        <v>8.561217405919038e-96</v>
       </c>
     </row>
     <row r="5">
@@ -2476,22 +2701,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0055</v>
+        <v>0.005</v>
       </c>
       <c r="C5" t="n">
         <v>0.0005</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1241</v>
+        <v>0.1108</v>
       </c>
       <c r="E5" t="n">
         <v>0.0108</v>
       </c>
       <c r="F5" t="n">
-        <v>11.4608</v>
+        <v>10.3036</v>
       </c>
       <c r="G5" t="n">
-        <v>2.07520829055946e-30</v>
+        <v>6.78429140847246e-25</v>
       </c>
     </row>
     <row r="6">
@@ -2501,22 +2726,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.0625</v>
+        <v>0.0562</v>
       </c>
       <c r="C6" t="n">
         <v>0.007900000000000001</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1145</v>
+        <v>0.1029</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0145</v>
+        <v>0.0144</v>
       </c>
       <c r="F6" t="n">
-        <v>7.9016</v>
+        <v>7.1263</v>
       </c>
       <c r="G6" t="n">
-        <v>2.753908328349476e-15</v>
+        <v>1.031254404489016e-12</v>
       </c>
     </row>
     <row r="7">
@@ -2526,22 +2751,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.0711</v>
+        <v>0.0594</v>
       </c>
       <c r="C7" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1221</v>
+        <v>0.102</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0151</v>
+        <v>0.015</v>
       </c>
       <c r="F7" t="n">
-        <v>8.096299999999999</v>
+        <v>6.8066</v>
       </c>
       <c r="G7" t="n">
-        <v>5.667406196789904e-16</v>
+        <v>9.990440825400547e-12</v>
       </c>
     </row>
     <row r="8">
@@ -2551,22 +2776,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.0674</v>
+        <v>0.0641</v>
       </c>
       <c r="C8" t="n">
-        <v>0.008200000000000001</v>
+        <v>0.0081</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0948</v>
+        <v>0.0901</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0115</v>
+        <v>0.0114</v>
       </c>
       <c r="F8" t="n">
-        <v>8.245100000000001</v>
+        <v>7.9224</v>
       </c>
       <c r="G8" t="n">
-        <v>1.650205533892556e-16</v>
+        <v>2.329922375313903e-15</v>
       </c>
     </row>
     <row r="9">
@@ -2576,22 +2801,22 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.0447</v>
+        <v>0.0453</v>
       </c>
       <c r="C9" t="n">
         <v>0.007900000000000001</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0553</v>
+        <v>0.056</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0098</v>
+        <v>0.0097</v>
       </c>
       <c r="F9" t="n">
-        <v>5.6326</v>
+        <v>5.755</v>
       </c>
       <c r="G9" t="n">
-        <v>1.775526925826283e-08</v>
+        <v>8.664252843529594e-09</v>
       </c>
     </row>
     <row r="10">
@@ -2601,22 +2826,22 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.1096</v>
+        <v>0.1042</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0104</v>
+        <v>0.0103</v>
       </c>
       <c r="D10" t="n">
-        <v>0.158</v>
+        <v>0.1501</v>
       </c>
       <c r="E10" t="n">
-        <v>0.015</v>
+        <v>0.0148</v>
       </c>
       <c r="F10" t="n">
-        <v>10.5436</v>
+        <v>10.1623</v>
       </c>
       <c r="G10" t="n">
-        <v>5.436701966806563e-26</v>
+        <v>2.919873706899104e-24</v>
       </c>
     </row>
     <row r="11">
@@ -2626,22 +2851,22 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0624</v>
+        <v>0.0616</v>
       </c>
       <c r="C11" t="n">
-        <v>0.008200000000000001</v>
+        <v>0.0081</v>
       </c>
       <c r="D11" t="n">
-        <v>0.08840000000000001</v>
+        <v>0.0872</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0116</v>
+        <v>0.0115</v>
       </c>
       <c r="F11" t="n">
-        <v>7.6405</v>
+        <v>7.575</v>
       </c>
       <c r="G11" t="n">
-        <v>2.16405738727976e-14</v>
+        <v>3.592642487954667e-14</v>
       </c>
     </row>
     <row r="12">
@@ -2651,22 +2876,22 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.07539999999999999</v>
+        <v>0.06809999999999999</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0103</v>
+        <v>0.0102</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0829</v>
+        <v>0.075</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0113</v>
+        <v>0.0112</v>
       </c>
       <c r="F12" t="n">
-        <v>7.3177</v>
+        <v>6.7122</v>
       </c>
       <c r="G12" t="n">
-        <v>2.523047702038281e-13</v>
+        <v>1.917366524943948e-11</v>
       </c>
     </row>
     <row r="13">
@@ -2676,22 +2901,22 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.0564</v>
+        <v>0.0504</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0086</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0668</v>
+        <v>0.0596</v>
       </c>
       <c r="E13" t="n">
-        <v>0.0101</v>
+        <v>0.01</v>
       </c>
       <c r="F13" t="n">
-        <v>6.5904</v>
+        <v>5.9328</v>
       </c>
       <c r="G13" t="n">
-        <v>4.387768640253819e-11</v>
+        <v>2.978592861436064e-09</v>
       </c>
     </row>
     <row r="14">
@@ -2701,22 +2926,22 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.0324</v>
+        <v>0.0321</v>
       </c>
       <c r="C14" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.0089</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0322</v>
+        <v>0.0319</v>
       </c>
       <c r="E14" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="F14" t="n">
-        <v>3.6002</v>
+        <v>3.621</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0003180129136090101</v>
+        <v>0.0002934666453694434</v>
       </c>
     </row>
     <row r="15">
@@ -2726,22 +2951,22 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.0106</v>
+        <v>0.0067</v>
       </c>
       <c r="C15" t="n">
-        <v>0.008399999999999999</v>
+        <v>0.0083</v>
       </c>
       <c r="D15" t="n">
-        <v>0.009299999999999999</v>
+        <v>0.0059</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0074</v>
+        <v>0.0073</v>
       </c>
       <c r="F15" t="n">
-        <v>1.2663</v>
+        <v>0.8081</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2054099506572642</v>
+        <v>0.4190591852696735</v>
       </c>
     </row>
     <row r="16">
@@ -2751,22 +2976,22 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.0273</v>
+        <v>0.0323</v>
       </c>
       <c r="C16" t="n">
-        <v>0.0086</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="D16" t="n">
-        <v>0.0245</v>
+        <v>0.029</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0077</v>
+        <v>0.0078</v>
       </c>
       <c r="F16" t="n">
-        <v>3.1736</v>
+        <v>3.7023</v>
       </c>
       <c r="G16" t="n">
-        <v>0.001505442893215186</v>
+        <v>0.000213681386164429</v>
       </c>
     </row>
     <row r="17">
@@ -2776,22 +3001,22 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.08790000000000001</v>
+        <v>0.07729999999999999</v>
       </c>
       <c r="C17" t="n">
-        <v>0.0173</v>
+        <v>0.0172</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0595</v>
+        <v>0.0523</v>
       </c>
       <c r="E17" t="n">
         <v>0.0117</v>
       </c>
       <c r="F17" t="n">
-        <v>5.0753</v>
+        <v>4.4864</v>
       </c>
       <c r="G17" t="n">
-        <v>3.868882024923099e-07</v>
+        <v>7.244521904004026e-06</v>
       </c>
     </row>
     <row r="18">
@@ -2801,22 +3026,22 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.0542</v>
+        <v>0.0414</v>
       </c>
       <c r="C18" t="n">
-        <v>0.0231</v>
+        <v>0.0227</v>
       </c>
       <c r="D18" t="n">
-        <v>0.0229</v>
+        <v>0.0175</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0097</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="F18" t="n">
-        <v>2.35</v>
+        <v>1.8233</v>
       </c>
       <c r="G18" t="n">
-        <v>0.01877297163093312</v>
+        <v>0.06825282942830668</v>
       </c>
     </row>
     <row r="19">
@@ -2826,22 +3051,22 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.0468</v>
+        <v>0.0309</v>
       </c>
       <c r="C19" t="n">
-        <v>0.0235</v>
+        <v>0.0236</v>
       </c>
       <c r="D19" t="n">
-        <v>0.014</v>
+        <v>0.0092</v>
       </c>
       <c r="E19" t="n">
-        <v>0.007</v>
+        <v>0.0071</v>
       </c>
       <c r="F19" t="n">
-        <v>1.992</v>
+        <v>1.307</v>
       </c>
       <c r="G19" t="n">
-        <v>0.046376110863128</v>
+        <v>0.1912086943180784</v>
       </c>
     </row>
     <row r="20">
@@ -2851,22 +3076,22 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-0.1022</v>
+        <v>-0.0955</v>
       </c>
       <c r="C20" t="n">
-        <v>0.005</v>
+        <v>0.0049</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.1997</v>
+        <v>-0.1867</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0097</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="F20" t="n">
-        <v>-20.5353</v>
+        <v>-19.4143</v>
       </c>
       <c r="G20" t="n">
-        <v>1.041834936009393e-93</v>
+        <v>5.839484225313443e-84</v>
       </c>
     </row>
     <row r="21">
@@ -2876,22 +3101,22 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-0.1019</v>
+        <v>-0.0973</v>
       </c>
       <c r="C21" t="n">
         <v>0.0054</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.1739</v>
+        <v>-0.166</v>
       </c>
       <c r="E21" t="n">
-        <v>0.009299999999999999</v>
+        <v>0.0092</v>
       </c>
       <c r="F21" t="n">
-        <v>-18.699</v>
+        <v>-18.0107</v>
       </c>
       <c r="G21" t="n">
-        <v>5.043982096799466e-78</v>
+        <v>1.605448232048225e-72</v>
       </c>
     </row>
     <row r="22">
@@ -2901,22 +3126,22 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>-0.1215</v>
+        <v>-0.1178</v>
       </c>
       <c r="C22" t="n">
-        <v>0.0073</v>
+        <v>0.0072</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.1596</v>
+        <v>-0.1548</v>
       </c>
       <c r="E22" t="n">
         <v>0.0095</v>
       </c>
       <c r="F22" t="n">
-        <v>-16.7415</v>
+        <v>-16.3596</v>
       </c>
       <c r="G22" t="n">
-        <v>6.526643723517673e-63</v>
+        <v>3.714453782580163e-60</v>
       </c>
     </row>
     <row r="23">
@@ -2926,22 +3151,22 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-0.0703</v>
+        <v>-0.0711</v>
       </c>
       <c r="C23" t="n">
-        <v>0.006</v>
+        <v>0.0059</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.1373</v>
+        <v>-0.1389</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0117</v>
+        <v>0.0116</v>
       </c>
       <c r="F23" t="n">
-        <v>-11.7732</v>
+        <v>-11.9933</v>
       </c>
       <c r="G23" t="n">
-        <v>5.362426103971977e-32</v>
+        <v>3.851077963661381e-33</v>
       </c>
     </row>
     <row r="24">
@@ -2951,22 +3176,97 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>-0.1014</v>
+        <v>-0.1016</v>
       </c>
       <c r="C24" t="n">
-        <v>0.0077</v>
+        <v>0.0076</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.1151</v>
+        <v>-0.1154</v>
       </c>
       <c r="E24" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.0086</v>
       </c>
       <c r="F24" t="n">
-        <v>-13.2099</v>
+        <v>-13.3482</v>
       </c>
       <c r="G24" t="n">
-        <v>7.692666028543185e-40</v>
+        <v>1.214058286056416e-40</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>d_aa</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>-0.046</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.0037</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-0.0864</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.0069</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-12.4908</v>
+      </c>
+      <c r="G25" t="n">
+        <v>8.380030162345431e-36</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>d_indie</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>-0.0306</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.0046</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-0.0453</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.0068</v>
+      </c>
+      <c r="F26" t="n">
+        <v>-6.6292</v>
+      </c>
+      <c r="G26" t="n">
+        <v>3.374381682041112e-11</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>d_unknown</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>-0.0586</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.0038</v>
+      </c>
+      <c r="D27" t="n">
+        <v>-0.08699999999999999</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.0057</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-15.2322</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2.162640598758015e-52</v>
       </c>
     </row>
   </sheetData>
@@ -2980,7 +3280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3027,7 +3327,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.0988</v>
+        <v>0.105</v>
       </c>
       <c r="C2" t="n">
         <v>0.0035</v>
@@ -3035,10 +3335,10 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>28.4091</v>
+        <v>29.6153</v>
       </c>
       <c r="G2" t="n">
-        <v>1.56071571869917e-177</v>
+        <v>9.493174009798496e-193</v>
       </c>
     </row>
     <row r="3">
@@ -3048,22 +3348,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.0259</v>
+        <v>0.025</v>
       </c>
       <c r="C3" t="n">
         <v>0.0016</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2115</v>
+        <v>0.2048</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0133</v>
+        <v>0.0132</v>
       </c>
       <c r="F3" t="n">
-        <v>15.9039</v>
+        <v>15.4752</v>
       </c>
       <c r="G3" t="n">
-        <v>5.952253279975866e-57</v>
+        <v>5.098290085572425e-54</v>
       </c>
     </row>
     <row r="4">
@@ -3073,22 +3373,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.0537</v>
+        <v>-0.0502</v>
       </c>
       <c r="C4" t="n">
         <v>0.0024</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.2596</v>
+        <v>-0.2425</v>
       </c>
       <c r="E4" t="n">
         <v>0.0117</v>
       </c>
       <c r="F4" t="n">
-        <v>-22.2787</v>
+        <v>-20.798</v>
       </c>
       <c r="G4" t="n">
-        <v>5.943237171671356e-110</v>
+        <v>4.516185900993735e-96</v>
       </c>
     </row>
     <row r="5">
@@ -3098,22 +3398,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0018</v>
+        <v>0.0017</v>
       </c>
       <c r="C5" t="n">
         <v>0.0002</v>
       </c>
       <c r="D5" t="n">
-        <v>0.09089999999999999</v>
+        <v>0.08749999999999999</v>
       </c>
       <c r="E5" t="n">
         <v>0.008699999999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>10.3999</v>
+        <v>10.1001</v>
       </c>
       <c r="G5" t="n">
-        <v>2.482206125847451e-25</v>
+        <v>5.520102026723362e-24</v>
       </c>
     </row>
     <row r="6">
@@ -3123,22 +3423,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.0266</v>
+        <v>0.0243</v>
       </c>
       <c r="C6" t="n">
         <v>0.0033</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1048</v>
+        <v>0.09569999999999999</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0129</v>
+        <v>0.0128</v>
       </c>
       <c r="F6" t="n">
-        <v>8.148</v>
+        <v>7.4661</v>
       </c>
       <c r="G6" t="n">
-        <v>3.698699617754467e-16</v>
+        <v>8.263638734334532e-14</v>
       </c>
     </row>
     <row r="7">
@@ -3148,22 +3448,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.0333</v>
+        <v>0.0286</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0035</v>
+        <v>0.0034</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1277</v>
+        <v>0.1095</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0133</v>
+        <v>0.0132</v>
       </c>
       <c r="F7" t="n">
-        <v>9.5997</v>
+        <v>8.3161</v>
       </c>
       <c r="G7" t="n">
-        <v>8.021169245052314e-22</v>
+        <v>9.090366403607607e-17</v>
       </c>
     </row>
     <row r="8">
@@ -3173,22 +3473,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.0325</v>
+        <v>0.0313</v>
       </c>
       <c r="C8" t="n">
         <v>0.0033</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1045</v>
+        <v>0.1006</v>
       </c>
       <c r="E8" t="n">
         <v>0.0106</v>
       </c>
       <c r="F8" t="n">
-        <v>9.822100000000001</v>
+        <v>9.5143</v>
       </c>
       <c r="G8" t="n">
-        <v>9.041266072722864e-23</v>
+        <v>1.828701716444621e-21</v>
       </c>
     </row>
     <row r="9">
@@ -3198,22 +3498,22 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.0202</v>
+        <v>0.021</v>
       </c>
       <c r="C9" t="n">
         <v>0.003</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0553</v>
+        <v>0.0576</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0083</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>6.6911</v>
+        <v>6.9861</v>
       </c>
       <c r="G9" t="n">
-        <v>2.214729568316151e-11</v>
+        <v>2.826954633779415e-12</v>
       </c>
     </row>
     <row r="10">
@@ -3223,22 +3523,22 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.0467</v>
+        <v>0.0449</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0047</v>
+        <v>0.0046</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1435</v>
+        <v>0.138</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0144</v>
+        <v>0.0142</v>
       </c>
       <c r="F10" t="n">
-        <v>9.936400000000001</v>
+        <v>9.6936</v>
       </c>
       <c r="G10" t="n">
-        <v>2.892208930517625e-23</v>
+        <v>3.210556741344724e-22</v>
       </c>
     </row>
     <row r="11">
@@ -3248,22 +3548,22 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0212</v>
+        <v>0.022</v>
       </c>
       <c r="C11" t="n">
         <v>0.0033</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0653</v>
+        <v>0.06759999999999999</v>
       </c>
       <c r="E11" t="n">
         <v>0.01</v>
       </c>
       <c r="F11" t="n">
-        <v>6.4986</v>
+        <v>6.7563</v>
       </c>
       <c r="G11" t="n">
-        <v>8.107322170513796e-11</v>
+        <v>1.415727937803293e-11</v>
       </c>
     </row>
     <row r="12">
@@ -3273,22 +3573,22 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.0276</v>
+        <v>0.0254</v>
       </c>
       <c r="C12" t="n">
         <v>0.0032</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0701</v>
+        <v>0.0645</v>
       </c>
       <c r="E12" t="n">
-        <v>0.008200000000000001</v>
+        <v>0.0081</v>
       </c>
       <c r="F12" t="n">
-        <v>8.539099999999999</v>
+        <v>7.9973</v>
       </c>
       <c r="G12" t="n">
-        <v>1.352622650770721e-17</v>
+        <v>1.271356955724793e-15</v>
       </c>
     </row>
     <row r="13">
@@ -3298,22 +3598,22 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.0206</v>
+        <v>0.0186</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0035</v>
+        <v>0.0034</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0522</v>
+        <v>0.0471</v>
       </c>
       <c r="E13" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="F13" t="n">
-        <v>5.9529</v>
+        <v>5.3959</v>
       </c>
       <c r="G13" t="n">
-        <v>2.63408016266086e-09</v>
+        <v>6.818386801856259e-08</v>
       </c>
     </row>
     <row r="14">
@@ -3323,22 +3623,22 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.0171</v>
+        <v>0.0174</v>
       </c>
       <c r="C14" t="n">
         <v>0.0038</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0362</v>
+        <v>0.0368</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0081</v>
+        <v>0.008</v>
       </c>
       <c r="F14" t="n">
-        <v>4.4642</v>
+        <v>4.6235</v>
       </c>
       <c r="G14" t="n">
-        <v>8.037893656124215e-06</v>
+        <v>3.774055178535852e-06</v>
       </c>
     </row>
     <row r="15">
@@ -3348,22 +3648,22 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.0049</v>
+        <v>0.0037</v>
       </c>
       <c r="C15" t="n">
         <v>0.003</v>
       </c>
       <c r="D15" t="n">
-        <v>0.0095</v>
+        <v>0.0073</v>
       </c>
       <c r="E15" t="n">
         <v>0.0059</v>
       </c>
       <c r="F15" t="n">
-        <v>1.6035</v>
+        <v>1.2452</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1088288734084694</v>
+        <v>0.2130499859921222</v>
       </c>
     </row>
     <row r="16">
@@ -3373,22 +3673,22 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.0149</v>
+        <v>0.0178</v>
       </c>
       <c r="C16" t="n">
         <v>0.0029</v>
       </c>
       <c r="D16" t="n">
-        <v>0.0307</v>
+        <v>0.0368</v>
       </c>
       <c r="E16" t="n">
-        <v>0.006</v>
+        <v>0.0061</v>
       </c>
       <c r="F16" t="n">
-        <v>5.14</v>
+        <v>6.0578</v>
       </c>
       <c r="G16" t="n">
-        <v>2.746841668685638e-07</v>
+        <v>1.379790101527942e-09</v>
       </c>
     </row>
     <row r="17">
@@ -3398,22 +3698,22 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.0298</v>
+        <v>0.0253</v>
       </c>
       <c r="C17" t="n">
         <v>0.0075</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0432</v>
+        <v>0.0368</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0109</v>
+        <v>0.0108</v>
       </c>
       <c r="F17" t="n">
-        <v>3.9666</v>
+        <v>3.3951</v>
       </c>
       <c r="G17" t="n">
-        <v>7.291393614817315e-05</v>
+        <v>0.0006860189959474789</v>
       </c>
     </row>
     <row r="18">
@@ -3423,22 +3723,22 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.0165</v>
+        <v>0.011</v>
       </c>
       <c r="C18" t="n">
-        <v>0.0071</v>
+        <v>0.0069</v>
       </c>
       <c r="D18" t="n">
-        <v>0.0158</v>
+        <v>0.0105</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0068</v>
+        <v>0.0067</v>
       </c>
       <c r="F18" t="n">
-        <v>2.3259</v>
+        <v>1.5783</v>
       </c>
       <c r="G18" t="n">
-        <v>0.02002286147083859</v>
+        <v>0.1145049998589514</v>
       </c>
     </row>
     <row r="19">
@@ -3448,22 +3748,22 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.0091</v>
+        <v>0.0015</v>
       </c>
       <c r="C19" t="n">
         <v>0.0074</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0063</v>
+        <v>0.001</v>
       </c>
       <c r="E19" t="n">
         <v>0.0051</v>
       </c>
       <c r="F19" t="n">
-        <v>1.2258</v>
+        <v>0.1989</v>
       </c>
       <c r="G19" t="n">
-        <v>0.2202888603984025</v>
+        <v>0.8423610967934463</v>
       </c>
     </row>
     <row r="20">
@@ -3473,22 +3773,22 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-0.0599</v>
+        <v>-0.0568</v>
       </c>
       <c r="C20" t="n">
         <v>0.0021</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.2679</v>
+        <v>-0.2539</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0094</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="F20" t="n">
-        <v>-28.3566</v>
+        <v>-27.4281</v>
       </c>
       <c r="G20" t="n">
-        <v>6.941543432780558e-177</v>
+        <v>1.267181109150088e-165</v>
       </c>
     </row>
     <row r="21">
@@ -3498,22 +3798,22 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-0.0587</v>
+        <v>-0.0563</v>
       </c>
       <c r="C21" t="n">
         <v>0.0023</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.2236</v>
+        <v>-0.2144</v>
       </c>
       <c r="E21" t="n">
-        <v>0.0089</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="F21" t="n">
-        <v>-25.22</v>
+        <v>-24.5696</v>
       </c>
       <c r="G21" t="n">
-        <v>2.418274690132437e-140</v>
+        <v>2.670911495138096e-133</v>
       </c>
     </row>
     <row r="22">
@@ -3523,22 +3823,22 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>-0.0725</v>
+        <v>-0.07140000000000001</v>
       </c>
       <c r="C22" t="n">
         <v>0.0027</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.198</v>
+        <v>-0.195</v>
       </c>
       <c r="E22" t="n">
-        <v>0.0075</v>
+        <v>0.0074</v>
       </c>
       <c r="F22" t="n">
-        <v>-26.3976</v>
+        <v>-26.2031</v>
       </c>
       <c r="G22" t="n">
-        <v>1.460463677895199e-153</v>
+        <v>2.452221048853129e-151</v>
       </c>
     </row>
     <row r="23">
@@ -3548,22 +3848,22 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-0.048</v>
+        <v>-0.0485</v>
       </c>
       <c r="C23" t="n">
         <v>0.0026</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.2043</v>
+        <v>-0.2064</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0112</v>
+        <v>0.0111</v>
       </c>
       <c r="F23" t="n">
-        <v>-18.2484</v>
+        <v>-18.5539</v>
       </c>
       <c r="G23" t="n">
-        <v>2.130127519517401e-74</v>
+        <v>7.578256781602136e-77</v>
       </c>
     </row>
     <row r="24">
@@ -3573,22 +3873,97 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>-0.0357</v>
+        <v>-0.0355</v>
       </c>
       <c r="C24" t="n">
-        <v>0.0038</v>
+        <v>0.0037</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.0921</v>
+        <v>-0.0917</v>
       </c>
       <c r="E24" t="n">
-        <v>0.0097</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="F24" t="n">
-        <v>-9.5046</v>
+        <v>-9.533200000000001</v>
       </c>
       <c r="G24" t="n">
-        <v>2.008450123393033e-21</v>
+        <v>1.525523201478916e-21</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>d_aa</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>-0.0183</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-0.0769</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.0061</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-12.6984</v>
+      </c>
+      <c r="G25" t="n">
+        <v>6.031610362271175e-37</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>d_indie</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>-0.0173</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.0018</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-0.0573</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.0058</v>
+      </c>
+      <c r="F26" t="n">
+        <v>-9.868</v>
+      </c>
+      <c r="G26" t="n">
+        <v>5.728423285631834e-23</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>d_unknown</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>-0.0245</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="D27" t="n">
+        <v>-0.0863</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.0054</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-15.8974</v>
+      </c>
+      <c r="G27" t="n">
+        <v>6.609746737921694e-57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update standardized coef to include percentages
</commit_message>
<xml_diff>
--- a/output/coefficients/standardized/standardized_ALL.xlsx
+++ b/output/coefficients/standardized/standardized_ALL.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -438,20 +438,25 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>pct_effect (%)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>SE_Beta</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>t</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>p</t>
         </is>
@@ -471,10 +476,11 @@
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
-      <c r="F2" t="n">
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
         <v>49.3949</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -491,15 +497,18 @@
         <v>0.0049</v>
       </c>
       <c r="D3" t="n">
+        <v>11.3631</v>
+      </c>
+      <c r="E3" t="n">
         <v>0.2328</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>0.0106</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>21.9733</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>5.19024484586208e-107</v>
       </c>
     </row>
@@ -516,15 +525,18 @@
         <v>0.0075</v>
       </c>
       <c r="D4" t="n">
+        <v>-21.771</v>
+      </c>
+      <c r="E4" t="n">
         <v>-0.3251</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>0.009900000000000001</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>-32.7927</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>7.492269383312129e-236</v>
       </c>
     </row>
@@ -541,15 +553,18 @@
         <v>0.0005</v>
       </c>
       <c r="D5" t="n">
+        <v>-0.1484</v>
+      </c>
+      <c r="E5" t="n">
         <v>-0.022</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>0.007900000000000001</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>-2.768</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>0.005640304136887425</v>
       </c>
     </row>
@@ -566,15 +581,18 @@
         <v>0.0091</v>
       </c>
       <c r="D6" t="n">
+        <v>5.4331</v>
+      </c>
+      <c r="E6" t="n">
         <v>0.0601</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>0.0103</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>5.8113</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>6.199053613937379e-09</v>
       </c>
     </row>
@@ -591,15 +609,18 @@
         <v>0.0097</v>
       </c>
       <c r="D7" t="n">
+        <v>7.3192</v>
+      </c>
+      <c r="E7" t="n">
         <v>0.07580000000000001</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>0.0104</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>7.2972</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>2.937960448986889e-13</v>
       </c>
     </row>
@@ -616,15 +637,18 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="D8" t="n">
+        <v>6.094</v>
+      </c>
+      <c r="E8" t="n">
         <v>0.0574</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>0.008800000000000001</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>6.5405</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>6.129438846606865e-11</v>
       </c>
     </row>
@@ -641,15 +665,18 @@
         <v>0.008200000000000001</v>
       </c>
       <c r="D9" t="n">
+        <v>0.9947</v>
+      </c>
+      <c r="E9" t="n">
         <v>0.009299999999999999</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>0.0077</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>1.2043</v>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>0.2284826860528429</v>
       </c>
     </row>
@@ -666,15 +693,18 @@
         <v>0.014</v>
       </c>
       <c r="D10" t="n">
+        <v>14.0269</v>
+      </c>
+      <c r="E10" t="n">
         <v>0.109</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>0.0116</v>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>9.3592</v>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>8.034314722850815e-21</v>
       </c>
     </row>
@@ -691,15 +721,18 @@
         <v>0.0104</v>
       </c>
       <c r="D11" t="n">
+        <v>4.5915</v>
+      </c>
+      <c r="E11" t="n">
         <v>0.0368</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>0.008500000000000001</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>4.3228</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>1.54082537388473e-05</v>
       </c>
     </row>
@@ -716,15 +749,18 @@
         <v>0.011</v>
       </c>
       <c r="D12" t="n">
+        <v>6.6348</v>
+      </c>
+      <c r="E12" t="n">
         <v>0.0473</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>0.0081</v>
       </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>5.8224</v>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>5.801343260495562e-09</v>
       </c>
     </row>
@@ -741,15 +777,18 @@
         <v>0.0116</v>
       </c>
       <c r="D13" t="n">
+        <v>4.436</v>
+      </c>
+      <c r="E13" t="n">
         <v>0.0295</v>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>0.007900000000000001</v>
       </c>
-      <c r="F13" t="n">
+      <c r="G13" t="n">
         <v>3.7416</v>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>0.0001828608945014619</v>
       </c>
     </row>
@@ -766,15 +805,18 @@
         <v>0.012</v>
       </c>
       <c r="D14" t="n">
+        <v>3.5321</v>
+      </c>
+      <c r="E14" t="n">
         <v>0.0219</v>
       </c>
-      <c r="E14" t="n">
+      <c r="F14" t="n">
         <v>0.0075</v>
       </c>
-      <c r="F14" t="n">
+      <c r="G14" t="n">
         <v>2.9029</v>
       </c>
-      <c r="G14" t="n">
+      <c r="H14" t="n">
         <v>0.003697766179605234</v>
       </c>
     </row>
@@ -791,15 +833,18 @@
         <v>0.0098</v>
       </c>
       <c r="D15" t="n">
+        <v>-3.8328</v>
+      </c>
+      <c r="E15" t="n">
         <v>-0.0231</v>
       </c>
-      <c r="E15" t="n">
+      <c r="F15" t="n">
         <v>0.0058</v>
       </c>
-      <c r="F15" t="n">
+      <c r="G15" t="n">
         <v>-3.9877</v>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
         <v>6.671685620093757e-05</v>
       </c>
     </row>
@@ -816,15 +861,18 @@
         <v>0.0106</v>
       </c>
       <c r="D16" t="n">
+        <v>1.192</v>
+      </c>
+      <c r="E16" t="n">
         <v>0.0068</v>
       </c>
-      <c r="E16" t="n">
+      <c r="F16" t="n">
         <v>0.006</v>
       </c>
-      <c r="F16" t="n">
+      <c r="G16" t="n">
         <v>1.1205</v>
       </c>
-      <c r="G16" t="n">
+      <c r="H16" t="n">
         <v>0.2625053442913986</v>
       </c>
     </row>
@@ -841,15 +889,18 @@
         <v>0.0232</v>
       </c>
       <c r="D17" t="n">
+        <v>9.547599999999999</v>
+      </c>
+      <c r="E17" t="n">
         <v>0.036</v>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>0.0091</v>
       </c>
-      <c r="F17" t="n">
+      <c r="G17" t="n">
         <v>3.9356</v>
       </c>
-      <c r="G17" t="n">
+      <c r="H17" t="n">
         <v>8.297693984728184e-05</v>
       </c>
     </row>
@@ -866,15 +917,18 @@
         <v>0.008800000000000001</v>
       </c>
       <c r="D18" t="n">
+        <v>-2.6251</v>
+      </c>
+      <c r="E18" t="n">
         <v>-0.0092</v>
       </c>
-      <c r="E18" t="n">
+      <c r="F18" t="n">
         <v>0.0031</v>
       </c>
-      <c r="F18" t="n">
+      <c r="G18" t="n">
         <v>-3.016</v>
       </c>
-      <c r="G18" t="n">
+      <c r="H18" t="n">
         <v>0.002561019149257387</v>
       </c>
     </row>
@@ -891,15 +945,18 @@
         <v>0.0246</v>
       </c>
       <c r="D19" t="n">
+        <v>6.2009</v>
+      </c>
+      <c r="E19" t="n">
         <v>0.0175</v>
       </c>
-      <c r="E19" t="n">
+      <c r="F19" t="n">
         <v>0.0071</v>
       </c>
-      <c r="F19" t="n">
+      <c r="G19" t="n">
         <v>2.4446</v>
       </c>
-      <c r="G19" t="n">
+      <c r="H19" t="n">
         <v>0.01450079799139041</v>
       </c>
     </row>
@@ -916,15 +973,18 @@
         <v>0.0309</v>
       </c>
       <c r="D20" t="n">
+        <v>1.6641</v>
+      </c>
+      <c r="E20" t="n">
         <v>0.0033</v>
       </c>
-      <c r="E20" t="n">
+      <c r="F20" t="n">
         <v>0.0062</v>
       </c>
-      <c r="F20" t="n">
+      <c r="G20" t="n">
         <v>0.5346</v>
       </c>
-      <c r="G20" t="n">
+      <c r="H20" t="n">
         <v>0.5928969351046378</v>
       </c>
     </row>
@@ -941,15 +1001,18 @@
         <v>0.043</v>
       </c>
       <c r="D21" t="n">
+        <v>-27.5435</v>
+      </c>
+      <c r="E21" t="n">
         <v>-0.0459</v>
       </c>
-      <c r="E21" t="n">
+      <c r="F21" t="n">
         <v>0.0061</v>
       </c>
-      <c r="F21" t="n">
+      <c r="G21" t="n">
         <v>-7.4914</v>
       </c>
-      <c r="G21" t="n">
+      <c r="H21" t="n">
         <v>6.812353441902274e-14</v>
       </c>
     </row>
@@ -966,15 +1029,18 @@
         <v>0.0059</v>
       </c>
       <c r="D22" t="n">
+        <v>-11.3218</v>
+      </c>
+      <c r="E22" t="n">
         <v>-0.1597</v>
       </c>
-      <c r="E22" t="n">
+      <c r="F22" t="n">
         <v>0.0078</v>
       </c>
-      <c r="F22" t="n">
+      <c r="G22" t="n">
         <v>-20.4092</v>
       </c>
-      <c r="G22" t="n">
+      <c r="H22" t="n">
         <v>1.385639557257553e-92</v>
       </c>
     </row>
@@ -991,15 +1057,18 @@
         <v>0.0074</v>
       </c>
       <c r="D23" t="n">
+        <v>-9.6835</v>
+      </c>
+      <c r="E23" t="n">
         <v>-0.1059</v>
       </c>
-      <c r="E23" t="n">
+      <c r="F23" t="n">
         <v>0.0076</v>
       </c>
-      <c r="F23" t="n">
+      <c r="G23" t="n">
         <v>-13.8522</v>
       </c>
-      <c r="G23" t="n">
+      <c r="H23" t="n">
         <v>1.233771683303811e-43</v>
       </c>
     </row>
@@ -1016,15 +1085,18 @@
         <v>0.009299999999999999</v>
       </c>
       <c r="D24" t="n">
+        <v>-20.8679</v>
+      </c>
+      <c r="E24" t="n">
         <v>-0.1699</v>
       </c>
-      <c r="E24" t="n">
+      <c r="F24" t="n">
         <v>0.0068</v>
       </c>
-      <c r="F24" t="n">
+      <c r="G24" t="n">
         <v>-25.0389</v>
       </c>
-      <c r="G24" t="n">
+      <c r="H24" t="n">
         <v>2.307580081083772e-138</v>
       </c>
     </row>
@@ -1041,15 +1113,18 @@
         <v>0.0081</v>
       </c>
       <c r="D25" t="n">
+        <v>-4.5599</v>
+      </c>
+      <c r="E25" t="n">
         <v>-0.0539</v>
       </c>
-      <c r="E25" t="n">
+      <c r="F25" t="n">
         <v>0.0094</v>
       </c>
-      <c r="F25" t="n">
+      <c r="G25" t="n">
         <v>-5.7408</v>
       </c>
-      <c r="G25" t="n">
+      <c r="H25" t="n">
         <v>9.422985697115229e-09</v>
       </c>
     </row>
@@ -1066,15 +1141,18 @@
         <v>0.0063</v>
       </c>
       <c r="D26" t="n">
+        <v>-13.8511</v>
+      </c>
+      <c r="E26" t="n">
         <v>-0.1507</v>
       </c>
-      <c r="E26" t="n">
+      <c r="F26" t="n">
         <v>0.0064</v>
       </c>
-      <c r="F26" t="n">
+      <c r="G26" t="n">
         <v>-23.6238</v>
       </c>
-      <c r="G26" t="n">
+      <c r="H26" t="n">
         <v>2.196787974340853e-123</v>
       </c>
     </row>
@@ -1091,15 +1169,18 @@
         <v>0.0052</v>
       </c>
       <c r="D27" t="n">
+        <v>-8.504799999999999</v>
+      </c>
+      <c r="E27" t="n">
         <v>-0.1091</v>
       </c>
-      <c r="E27" t="n">
+      <c r="F27" t="n">
         <v>0.0064</v>
       </c>
-      <c r="F27" t="n">
+      <c r="G27" t="n">
         <v>-17.0953</v>
       </c>
-      <c r="G27" t="n">
+      <c r="H27" t="n">
         <v>1.609484180381554e-65</v>
       </c>
     </row>
@@ -1116,15 +1197,18 @@
         <v>0.0066</v>
       </c>
       <c r="D28" t="n">
+        <v>-6.2948</v>
+      </c>
+      <c r="E28" t="n">
         <v>-0.0611</v>
       </c>
-      <c r="E28" t="n">
+      <c r="F28" t="n">
         <v>0.0062</v>
       </c>
-      <c r="F28" t="n">
+      <c r="G28" t="n">
         <v>-9.814500000000001</v>
       </c>
-      <c r="G28" t="n">
+      <c r="H28" t="n">
         <v>9.7508750172815e-23</v>
       </c>
     </row>
@@ -1141,15 +1225,18 @@
         <v>0.0047</v>
       </c>
       <c r="D29" t="n">
+        <v>-12.49</v>
+      </c>
+      <c r="E29" t="n">
         <v>-0.1503</v>
       </c>
-      <c r="E29" t="n">
+      <c r="F29" t="n">
         <v>0.0053</v>
       </c>
-      <c r="F29" t="n">
+      <c r="G29" t="n">
         <v>-28.5691</v>
       </c>
-      <c r="G29" t="n">
+      <c r="H29" t="n">
         <v>1.627152312090757e-179</v>
       </c>
     </row>
@@ -1164,7 +1251,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1185,20 +1272,25 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>pct_effect (%)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>SE_Beta</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>t</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>p</t>
         </is>
@@ -1218,10 +1310,11 @@
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
-      <c r="F2" t="n">
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
         <v>32.7004</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>1.543351766214401e-234</v>
       </c>
     </row>
@@ -1238,15 +1331,18 @@
         <v>0.0038</v>
       </c>
       <c r="D3" t="n">
+        <v>7.8549</v>
+      </c>
+      <c r="E3" t="n">
         <v>0.2483</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>0.0126</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>19.645</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>6.379495164655918e-86</v>
       </c>
     </row>
@@ -1263,15 +1359,18 @@
         <v>0.006</v>
       </c>
       <c r="D4" t="n">
+        <v>-13.269</v>
+      </c>
+      <c r="E4" t="n">
         <v>-0.2726</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>0.0114</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>-23.8748</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>5.600838401538451e-126</v>
       </c>
     </row>
@@ -1288,15 +1387,18 @@
         <v>0.0005</v>
       </c>
       <c r="D5" t="n">
+        <v>-0.1727</v>
+      </c>
+      <c r="E5" t="n">
         <v>-0.0341</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>0.0091</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>-3.7688</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>0.0001640347282356813</v>
       </c>
     </row>
@@ -1313,15 +1415,18 @@
         <v>0.0092</v>
       </c>
       <c r="D6" t="n">
+        <v>5.6277</v>
+      </c>
+      <c r="E6" t="n">
         <v>0.0852</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>0.0144</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>5.9339</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>2.957447492894423e-09</v>
       </c>
     </row>
@@ -1338,15 +1443,18 @@
         <v>0.0094</v>
       </c>
       <c r="D7" t="n">
+        <v>6.5406</v>
+      </c>
+      <c r="E7" t="n">
         <v>0.0949</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>0.0141</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>6.7219</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>1.79366847143131e-11</v>
       </c>
     </row>
@@ -1363,15 +1471,18 @@
         <v>0.0097</v>
       </c>
       <c r="D8" t="n">
+        <v>7.5972</v>
+      </c>
+      <c r="E8" t="n">
         <v>0.0911</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>0.012</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>7.5619</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>3.972147382998328e-14</v>
       </c>
     </row>
@@ -1388,15 +1499,18 @@
         <v>0.0095</v>
       </c>
       <c r="D9" t="n">
+        <v>3.543</v>
+      </c>
+      <c r="E9" t="n">
         <v>0.0363</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>0.009900000000000001</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>3.6551</v>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>0.0002570401520009639</v>
       </c>
     </row>
@@ -1413,15 +1527,18 @@
         <v>0.0124</v>
       </c>
       <c r="D10" t="n">
+        <v>11.1497</v>
+      </c>
+      <c r="E10" t="n">
         <v>0.129</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>0.0151</v>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>8.5166</v>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>1.643557135152196e-17</v>
       </c>
     </row>
@@ -1438,15 +1555,18 @@
         <v>0.0095</v>
       </c>
       <c r="D11" t="n">
+        <v>2.5858</v>
+      </c>
+      <c r="E11" t="n">
         <v>0.0308</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>0.0114</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>2.7004</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>0.006924581632716168</v>
       </c>
     </row>
@@ -1463,15 +1583,18 @@
         <v>0.0108</v>
       </c>
       <c r="D12" t="n">
+        <v>7.216</v>
+      </c>
+      <c r="E12" t="n">
         <v>0.0672</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>0.0104</v>
       </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>6.4358</v>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>1.228204934607188e-10</v>
       </c>
     </row>
@@ -1488,15 +1611,18 @@
         <v>0.009900000000000001</v>
       </c>
       <c r="D13" t="n">
+        <v>3.1426</v>
+      </c>
+      <c r="E13" t="n">
         <v>0.0314</v>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>0.01</v>
       </c>
-      <c r="F13" t="n">
+      <c r="G13" t="n">
         <v>3.1219</v>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>0.001796715394070818</v>
       </c>
     </row>
@@ -1513,15 +1639,18 @@
         <v>0.0116</v>
       </c>
       <c r="D14" t="n">
+        <v>5.7034</v>
+      </c>
+      <c r="E14" t="n">
         <v>0.0466</v>
       </c>
-      <c r="E14" t="n">
+      <c r="F14" t="n">
         <v>0.0098</v>
       </c>
-      <c r="F14" t="n">
+      <c r="G14" t="n">
         <v>4.7745</v>
       </c>
-      <c r="G14" t="n">
+      <c r="H14" t="n">
         <v>1.801970706125262e-06</v>
       </c>
     </row>
@@ -1538,15 +1667,18 @@
         <v>0.0105</v>
       </c>
       <c r="D15" t="n">
+        <v>-3.0229</v>
+      </c>
+      <c r="E15" t="n">
         <v>-0.021</v>
       </c>
-      <c r="E15" t="n">
+      <c r="F15" t="n">
         <v>0.0072</v>
       </c>
-      <c r="F15" t="n">
+      <c r="G15" t="n">
         <v>-2.9153</v>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
         <v>0.003553300905034483</v>
       </c>
     </row>
@@ -1563,15 +1695,18 @@
         <v>0.0102</v>
       </c>
       <c r="D16" t="n">
+        <v>1.7245</v>
+      </c>
+      <c r="E16" t="n">
         <v>0.0134</v>
       </c>
-      <c r="E16" t="n">
+      <c r="F16" t="n">
         <v>0.008</v>
       </c>
-      <c r="F16" t="n">
+      <c r="G16" t="n">
         <v>1.6731</v>
       </c>
-      <c r="G16" t="n">
+      <c r="H16" t="n">
         <v>0.09430899476652224</v>
       </c>
     </row>
@@ -1588,15 +1723,18 @@
         <v>0.0185</v>
       </c>
       <c r="D17" t="n">
+        <v>5.2294</v>
+      </c>
+      <c r="E17" t="n">
         <v>0.0288</v>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>0.0104</v>
       </c>
-      <c r="F17" t="n">
+      <c r="G17" t="n">
         <v>2.7568</v>
       </c>
-      <c r="G17" t="n">
+      <c r="H17" t="n">
         <v>0.005836821367813983</v>
       </c>
     </row>
@@ -1613,15 +1751,18 @@
         <v>0.025</v>
       </c>
       <c r="D18" t="n">
+        <v>5.6888</v>
+      </c>
+      <c r="E18" t="n">
         <v>0.0207</v>
       </c>
-      <c r="E18" t="n">
+      <c r="F18" t="n">
         <v>0.009299999999999999</v>
       </c>
-      <c r="F18" t="n">
+      <c r="G18" t="n">
         <v>2.2126</v>
       </c>
-      <c r="G18" t="n">
+      <c r="H18" t="n">
         <v>0.02692379429928699</v>
       </c>
     </row>
@@ -1638,15 +1779,18 @@
         <v>0.0228</v>
       </c>
       <c r="D19" t="n">
+        <v>0.9001</v>
+      </c>
+      <c r="E19" t="n">
         <v>0.0024</v>
       </c>
-      <c r="E19" t="n">
+      <c r="F19" t="n">
         <v>0.0062</v>
       </c>
-      <c r="F19" t="n">
+      <c r="G19" t="n">
         <v>0.3923</v>
       </c>
-      <c r="G19" t="n">
+      <c r="H19" t="n">
         <v>0.6948626568191176</v>
       </c>
     </row>
@@ -1663,15 +1807,18 @@
         <v>0.0051</v>
       </c>
       <c r="D20" t="n">
+        <v>-4.9144</v>
+      </c>
+      <c r="E20" t="n">
         <v>-0.08840000000000001</v>
       </c>
-      <c r="E20" t="n">
+      <c r="F20" t="n">
         <v>0.008999999999999999</v>
       </c>
-      <c r="F20" t="n">
+      <c r="G20" t="n">
         <v>-9.8391</v>
       </c>
-      <c r="G20" t="n">
+      <c r="H20" t="n">
         <v>7.639268626007967e-23</v>
       </c>
     </row>
@@ -1688,15 +1835,18 @@
         <v>0.0059</v>
       </c>
       <c r="D21" t="n">
+        <v>-3.5182</v>
+      </c>
+      <c r="E21" t="n">
         <v>-0.054</v>
       </c>
-      <c r="E21" t="n">
+      <c r="F21" t="n">
         <v>0.008999999999999999</v>
       </c>
-      <c r="F21" t="n">
+      <c r="G21" t="n">
         <v>-6.0283</v>
       </c>
-      <c r="G21" t="n">
+      <c r="H21" t="n">
         <v>1.657370377219674e-09</v>
       </c>
     </row>
@@ -1713,15 +1863,18 @@
         <v>0.0119</v>
       </c>
       <c r="D22" t="n">
+        <v>-14.7318</v>
+      </c>
+      <c r="E22" t="n">
         <v>-0.113</v>
       </c>
-      <c r="E22" t="n">
+      <c r="F22" t="n">
         <v>0.008399999999999999</v>
       </c>
-      <c r="F22" t="n">
+      <c r="G22" t="n">
         <v>-13.3933</v>
       </c>
-      <c r="G22" t="n">
+      <c r="H22" t="n">
         <v>6.61841632152771e-41</v>
       </c>
     </row>
@@ -1738,15 +1891,18 @@
         <v>0.0066</v>
       </c>
       <c r="D23" t="n">
+        <v>0.6251</v>
+      </c>
+      <c r="E23" t="n">
         <v>0.0106</v>
       </c>
-      <c r="E23" t="n">
+      <c r="F23" t="n">
         <v>0.0113</v>
       </c>
-      <c r="F23" t="n">
+      <c r="G23" t="n">
         <v>0.9374</v>
       </c>
-      <c r="G23" t="n">
+      <c r="H23" t="n">
         <v>0.3485507775861378</v>
       </c>
     </row>
@@ -1763,15 +1919,18 @@
         <v>0.0065</v>
       </c>
       <c r="D24" t="n">
+        <v>-9.8827</v>
+      </c>
+      <c r="E24" t="n">
         <v>-0.1059</v>
       </c>
-      <c r="E24" t="n">
+      <c r="F24" t="n">
         <v>0.0066</v>
       </c>
-      <c r="F24" t="n">
+      <c r="G24" t="n">
         <v>-16.0391</v>
       </c>
-      <c r="G24" t="n">
+      <c r="H24" t="n">
         <v>6.812758172713022e-58</v>
       </c>
     </row>
@@ -1788,15 +1947,18 @@
         <v>0.0046</v>
       </c>
       <c r="D25" t="n">
+        <v>-5.802</v>
+      </c>
+      <c r="E25" t="n">
         <v>-0.1001</v>
       </c>
-      <c r="E25" t="n">
+      <c r="F25" t="n">
         <v>0.0077</v>
       </c>
-      <c r="F25" t="n">
+      <c r="G25" t="n">
         <v>-13.0236</v>
       </c>
-      <c r="G25" t="n">
+      <c r="H25" t="n">
         <v>8.988103653279595e-39</v>
       </c>
     </row>
@@ -1813,15 +1975,18 @@
         <v>0.0059</v>
       </c>
       <c r="D26" t="n">
+        <v>-4.1795</v>
+      </c>
+      <c r="E26" t="n">
         <v>-0.0538</v>
       </c>
-      <c r="E26" t="n">
+      <c r="F26" t="n">
         <v>0.0075</v>
       </c>
-      <c r="F26" t="n">
+      <c r="G26" t="n">
         <v>-7.2129</v>
       </c>
-      <c r="G26" t="n">
+      <c r="H26" t="n">
         <v>5.477667856739737e-13</v>
       </c>
     </row>
@@ -1838,15 +2003,18 @@
         <v>0.005</v>
       </c>
       <c r="D27" t="n">
+        <v>-9.2737</v>
+      </c>
+      <c r="E27" t="n">
         <v>-0.1273</v>
       </c>
-      <c r="E27" t="n">
+      <c r="F27" t="n">
         <v>0.0066</v>
       </c>
-      <c r="F27" t="n">
+      <c r="G27" t="n">
         <v>-19.3015</v>
       </c>
-      <c r="G27" t="n">
+      <c r="H27" t="n">
         <v>5.21533632665722e-83</v>
       </c>
     </row>
@@ -1861,7 +2029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1882,20 +2050,25 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>pct_effect (%)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>SE_Beta</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>t</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>p</t>
         </is>
@@ -1915,10 +2088,11 @@
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
-      <c r="F2" t="n">
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
         <v>24.0928</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>2.973277728886143e-128</v>
       </c>
     </row>
@@ -1935,15 +2109,18 @@
         <v>0.0025</v>
       </c>
       <c r="D3" t="n">
+        <v>1.1707</v>
+      </c>
+      <c r="E3" t="n">
         <v>0.06759999999999999</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>0.0147</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>4.6011</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>4.201972236188619e-06</v>
       </c>
     </row>
@@ -1960,15 +2137,18 @@
         <v>0.0037</v>
       </c>
       <c r="D4" t="n">
+        <v>-1.3324</v>
+      </c>
+      <c r="E4" t="n">
         <v>-0.0565</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>0.0156</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>-3.6109</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>0.0003051525889843639</v>
       </c>
     </row>
@@ -1985,15 +2165,18 @@
         <v>0.0004</v>
       </c>
       <c r="D5" t="n">
+        <v>-0.4294</v>
+      </c>
+      <c r="E5" t="n">
         <v>-0.1965</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>0.016</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>-12.2809</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>1.147278220178956e-34</v>
       </c>
     </row>
@@ -2010,15 +2193,18 @@
         <v>0.0051</v>
       </c>
       <c r="D6" t="n">
+        <v>-2.7271</v>
+      </c>
+      <c r="E6" t="n">
         <v>-0.0999</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>0.0183</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>-5.4657</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>4.610764476576635e-08</v>
       </c>
     </row>
@@ -2035,15 +2221,18 @@
         <v>0.007</v>
       </c>
       <c r="D7" t="n">
+        <v>-1.4355</v>
+      </c>
+      <c r="E7" t="n">
         <v>-0.0416</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>0.0202</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>-2.0558</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>0.03979982084358254</v>
       </c>
     </row>
@@ -2060,15 +2249,18 @@
         <v>0.0058</v>
       </c>
       <c r="D8" t="n">
+        <v>-2.7297</v>
+      </c>
+      <c r="E8" t="n">
         <v>-0.0824</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>0.0173</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>-4.7519</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>2.015223998359697e-06</v>
       </c>
     </row>
@@ -2085,15 +2277,18 @@
         <v>0.0044</v>
       </c>
       <c r="D9" t="n">
+        <v>-4.8335</v>
+      </c>
+      <c r="E9" t="n">
         <v>-0.1734</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>0.0153</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>-11.3685</v>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>6.003318545909891e-30</v>
       </c>
     </row>
@@ -2110,15 +2305,18 @@
         <v>0.006</v>
       </c>
       <c r="D10" t="n">
+        <v>-4.2972</v>
+      </c>
+      <c r="E10" t="n">
         <v>-0.107</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>0.0147</v>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>-7.2786</v>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>3.37288044545696e-13</v>
       </c>
     </row>
@@ -2135,15 +2333,18 @@
         <v>0.0061</v>
       </c>
       <c r="D11" t="n">
+        <v>-6.8415</v>
+      </c>
+      <c r="E11" t="n">
         <v>-0.1281</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>0.011</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>-11.6207</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>3.233128502358928e-31</v>
       </c>
     </row>
@@ -2160,15 +2361,18 @@
         <v>0.0072</v>
       </c>
       <c r="D12" t="n">
+        <v>-3.382</v>
+      </c>
+      <c r="E12" t="n">
         <v>-0.0732</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>0.0154</v>
       </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>-4.7625</v>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>1.91211945963566e-06</v>
       </c>
     </row>
@@ -2185,15 +2389,18 @@
         <v>0.0091</v>
       </c>
       <c r="D13" t="n">
+        <v>-4.2974</v>
+      </c>
+      <c r="E13" t="n">
         <v>-0.0704</v>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>0.0146</v>
       </c>
-      <c r="F13" t="n">
+      <c r="G13" t="n">
         <v>-4.8254</v>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>1.397440453692042e-06</v>
       </c>
     </row>
@@ -2210,15 +2417,18 @@
         <v>0.006</v>
       </c>
       <c r="D14" t="n">
+        <v>-2.8998</v>
+      </c>
+      <c r="E14" t="n">
         <v>-0.0711</v>
       </c>
-      <c r="E14" t="n">
+      <c r="F14" t="n">
         <v>0.0146</v>
       </c>
-      <c r="F14" t="n">
+      <c r="G14" t="n">
         <v>-4.8768</v>
       </c>
-      <c r="G14" t="n">
+      <c r="H14" t="n">
         <v>1.078040353427481e-06</v>
       </c>
     </row>
@@ -2235,15 +2445,18 @@
         <v>0.008500000000000001</v>
       </c>
       <c r="D15" t="n">
+        <v>-1.5434</v>
+      </c>
+      <c r="E15" t="n">
         <v>-0.0295</v>
       </c>
-      <c r="E15" t="n">
+      <c r="F15" t="n">
         <v>0.0161</v>
       </c>
-      <c r="F15" t="n">
+      <c r="G15" t="n">
         <v>-1.8283</v>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
         <v>0.06750116419621574</v>
       </c>
     </row>
@@ -2260,15 +2473,18 @@
         <v>0.0086</v>
       </c>
       <c r="D16" t="n">
+        <v>-4.0339</v>
+      </c>
+      <c r="E16" t="n">
         <v>-0.0577</v>
       </c>
-      <c r="E16" t="n">
+      <c r="F16" t="n">
         <v>0.012</v>
       </c>
-      <c r="F16" t="n">
+      <c r="G16" t="n">
         <v>-4.7911</v>
       </c>
-      <c r="G16" t="n">
+      <c r="H16" t="n">
         <v>1.658427009483529e-06</v>
       </c>
     </row>
@@ -2285,15 +2501,18 @@
         <v>0.007</v>
       </c>
       <c r="D17" t="n">
+        <v>-4.1165</v>
+      </c>
+      <c r="E17" t="n">
         <v>-0.0535</v>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>0.0089</v>
       </c>
-      <c r="F17" t="n">
+      <c r="G17" t="n">
         <v>-6.0261</v>
       </c>
-      <c r="G17" t="n">
+      <c r="H17" t="n">
         <v>1.679855939870908e-09</v>
       </c>
     </row>
@@ -2310,15 +2529,18 @@
         <v>0.0044</v>
       </c>
       <c r="D18" t="n">
+        <v>-3.6839</v>
+      </c>
+      <c r="E18" t="n">
         <v>-0.068</v>
       </c>
-      <c r="E18" t="n">
+      <c r="F18" t="n">
         <v>0.008</v>
       </c>
-      <c r="F18" t="n">
+      <c r="G18" t="n">
         <v>-8.5556</v>
       </c>
-      <c r="G18" t="n">
+      <c r="H18" t="n">
         <v>1.172793169560562e-17</v>
       </c>
     </row>
@@ -2335,15 +2557,18 @@
         <v>0.0161</v>
       </c>
       <c r="D19" t="n">
+        <v>1.8218</v>
+      </c>
+      <c r="E19" t="n">
         <v>0.0169</v>
       </c>
-      <c r="E19" t="n">
+      <c r="F19" t="n">
         <v>0.0151</v>
       </c>
-      <c r="F19" t="n">
+      <c r="G19" t="n">
         <v>1.1194</v>
       </c>
-      <c r="G19" t="n">
+      <c r="H19" t="n">
         <v>0.2629609945769958</v>
       </c>
     </row>
@@ -2360,15 +2585,18 @@
         <v>0.0245</v>
       </c>
       <c r="D20" t="n">
+        <v>1.5893</v>
+      </c>
+      <c r="E20" t="n">
         <v>0.0105</v>
       </c>
-      <c r="E20" t="n">
+      <c r="F20" t="n">
         <v>0.0163</v>
       </c>
-      <c r="F20" t="n">
+      <c r="G20" t="n">
         <v>0.6433</v>
       </c>
-      <c r="G20" t="n">
+      <c r="H20" t="n">
         <v>0.5200393055702741</v>
       </c>
     </row>
@@ -2385,15 +2613,18 @@
         <v>0.0162</v>
       </c>
       <c r="D21" t="n">
+        <v>-0.8559</v>
+      </c>
+      <c r="E21" t="n">
         <v>-0.0065</v>
       </c>
-      <c r="E21" t="n">
+      <c r="F21" t="n">
         <v>0.0121</v>
       </c>
-      <c r="F21" t="n">
+      <c r="G21" t="n">
         <v>-0.5315</v>
       </c>
-      <c r="G21" t="n">
+      <c r="H21" t="n">
         <v>0.5950808586216669</v>
       </c>
     </row>
@@ -2410,15 +2641,18 @@
         <v>0.0037</v>
       </c>
       <c r="D22" t="n">
+        <v>0.2304</v>
+      </c>
+      <c r="E22" t="n">
         <v>0.009900000000000001</v>
       </c>
-      <c r="E22" t="n">
+      <c r="F22" t="n">
         <v>0.016</v>
       </c>
-      <c r="F22" t="n">
+      <c r="G22" t="n">
         <v>0.6157</v>
       </c>
-      <c r="G22" t="n">
+      <c r="H22" t="n">
         <v>0.5381087955485305</v>
       </c>
     </row>
@@ -2435,15 +2669,18 @@
         <v>0.0053</v>
       </c>
       <c r="D23" t="n">
+        <v>-2.6282</v>
+      </c>
+      <c r="E23" t="n">
         <v>-0.065</v>
       </c>
-      <c r="E23" t="n">
+      <c r="F23" t="n">
         <v>0.013</v>
       </c>
-      <c r="F23" t="n">
+      <c r="G23" t="n">
         <v>-4.9926</v>
       </c>
-      <c r="G23" t="n">
+      <c r="H23" t="n">
         <v>5.955884042550342e-07</v>
       </c>
     </row>
@@ -2460,15 +2697,18 @@
         <v>0.0034</v>
       </c>
       <c r="D24" t="n">
+        <v>-6.934</v>
+      </c>
+      <c r="E24" t="n">
         <v>-0.2017</v>
       </c>
-      <c r="E24" t="n">
+      <c r="F24" t="n">
         <v>0.009599999999999999</v>
       </c>
-      <c r="F24" t="n">
+      <c r="G24" t="n">
         <v>-20.9874</v>
       </c>
-      <c r="G24" t="n">
+      <c r="H24" t="n">
         <v>8.549389740776044e-98</v>
       </c>
     </row>
@@ -2485,15 +2725,18 @@
         <v>0.0029</v>
       </c>
       <c r="D25" t="n">
+        <v>-1.2938</v>
+      </c>
+      <c r="E25" t="n">
         <v>-0.0557</v>
       </c>
-      <c r="E25" t="n">
+      <c r="F25" t="n">
         <v>0.0125</v>
       </c>
-      <c r="F25" t="n">
+      <c r="G25" t="n">
         <v>-4.4549</v>
       </c>
-      <c r="G25" t="n">
+      <c r="H25" t="n">
         <v>8.392923020292335e-06</v>
       </c>
     </row>
@@ -2510,15 +2753,18 @@
         <v>0.0033</v>
       </c>
       <c r="D26" t="n">
+        <v>-3.0109</v>
+      </c>
+      <c r="E26" t="n">
         <v>-0.1157</v>
       </c>
-      <c r="E26" t="n">
+      <c r="F26" t="n">
         <v>0.0124</v>
       </c>
-      <c r="F26" t="n">
+      <c r="G26" t="n">
         <v>-9.331</v>
       </c>
-      <c r="G26" t="n">
+      <c r="H26" t="n">
         <v>1.048921794262594e-20</v>
       </c>
     </row>
@@ -2535,15 +2781,18 @@
         <v>0.0038</v>
       </c>
       <c r="D27" t="n">
+        <v>-3.6078</v>
+      </c>
+      <c r="E27" t="n">
         <v>-0.0926</v>
       </c>
-      <c r="E27" t="n">
+      <c r="F27" t="n">
         <v>0.0095</v>
       </c>
-      <c r="F27" t="n">
+      <c r="G27" t="n">
         <v>-9.7531</v>
       </c>
-      <c r="G27" t="n">
+      <c r="H27" t="n">
         <v>1.78922769219574e-22</v>
       </c>
     </row>
@@ -2560,15 +2809,18 @@
         <v>0.0033</v>
       </c>
       <c r="D28" t="n">
+        <v>-3.6778</v>
+      </c>
+      <c r="E28" t="n">
         <v>-0.141</v>
       </c>
-      <c r="E28" t="n">
+      <c r="F28" t="n">
         <v>0.0123</v>
       </c>
-      <c r="F28" t="n">
+      <c r="G28" t="n">
         <v>-11.4551</v>
       </c>
-      <c r="G28" t="n">
+      <c r="H28" t="n">
         <v>2.21591782514193e-30</v>
       </c>
     </row>
@@ -2583,7 +2835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2604,20 +2856,25 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>pct_effect (%)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>SE_Beta</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>t</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>p</t>
         </is>
@@ -2637,10 +2894,11 @@
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
-      <c r="F2" t="n">
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
         <v>29.5134</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>1.935312902244293e-191</v>
       </c>
     </row>
@@ -2657,15 +2915,18 @@
         <v>0.0033</v>
       </c>
       <c r="D3" t="n">
+        <v>5.7706</v>
+      </c>
+      <c r="E3" t="n">
         <v>0.2184</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>0.0129</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>16.9424</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>2.188213823860349e-64</v>
       </c>
     </row>
@@ -2682,15 +2943,18 @@
         <v>0.0053</v>
       </c>
       <c r="D4" t="n">
+        <v>-10.3385</v>
+      </c>
+      <c r="E4" t="n">
         <v>-0.2465</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>0.0119</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>-20.7673</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>8.561217405919038e-96</v>
       </c>
     </row>
@@ -2707,15 +2971,18 @@
         <v>0.0005</v>
       </c>
       <c r="D5" t="n">
+        <v>0.4965</v>
+      </c>
+      <c r="E5" t="n">
         <v>0.1108</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>0.0108</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>10.3036</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>6.78429140847246e-25</v>
       </c>
     </row>
@@ -2732,15 +2999,18 @@
         <v>0.007900000000000001</v>
       </c>
       <c r="D6" t="n">
+        <v>5.7773</v>
+      </c>
+      <c r="E6" t="n">
         <v>0.1029</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>0.0144</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>7.1263</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>1.031254404489016e-12</v>
       </c>
     </row>
@@ -2757,15 +3027,18 @@
         <v>0.008699999999999999</v>
       </c>
       <c r="D7" t="n">
+        <v>6.1204</v>
+      </c>
+      <c r="E7" t="n">
         <v>0.102</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>0.015</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>6.8066</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>9.990440825400547e-12</v>
       </c>
     </row>
@@ -2782,15 +3055,18 @@
         <v>0.0081</v>
       </c>
       <c r="D8" t="n">
+        <v>6.6191</v>
+      </c>
+      <c r="E8" t="n">
         <v>0.0901</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>0.0114</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>7.9224</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>2.329922375313903e-15</v>
       </c>
     </row>
@@ -2807,15 +3083,18 @@
         <v>0.007900000000000001</v>
       </c>
       <c r="D9" t="n">
+        <v>4.6327</v>
+      </c>
+      <c r="E9" t="n">
         <v>0.056</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>0.0097</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>5.755</v>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>8.664252843529594e-09</v>
       </c>
     </row>
@@ -2832,15 +3111,18 @@
         <v>0.0103</v>
       </c>
       <c r="D10" t="n">
+        <v>10.9795</v>
+      </c>
+      <c r="E10" t="n">
         <v>0.1501</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>0.0148</v>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>10.1623</v>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>2.919873706899104e-24</v>
       </c>
     </row>
@@ -2857,15 +3139,18 @@
         <v>0.0081</v>
       </c>
       <c r="D11" t="n">
+        <v>6.3586</v>
+      </c>
+      <c r="E11" t="n">
         <v>0.0872</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>0.0115</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>7.575</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>3.592642487954667e-14</v>
       </c>
     </row>
@@ -2882,15 +3167,18 @@
         <v>0.0102</v>
       </c>
       <c r="D12" t="n">
+        <v>7.0522</v>
+      </c>
+      <c r="E12" t="n">
         <v>0.075</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>0.0112</v>
       </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>6.7122</v>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>1.917366524943948e-11</v>
       </c>
     </row>
@@ -2907,15 +3195,18 @@
         <v>0.008500000000000001</v>
       </c>
       <c r="D13" t="n">
+        <v>5.166</v>
+      </c>
+      <c r="E13" t="n">
         <v>0.0596</v>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>0.01</v>
       </c>
-      <c r="F13" t="n">
+      <c r="G13" t="n">
         <v>5.9328</v>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>2.978592861436064e-09</v>
       </c>
     </row>
@@ -2932,15 +3223,18 @@
         <v>0.0089</v>
       </c>
       <c r="D14" t="n">
+        <v>3.2599</v>
+      </c>
+      <c r="E14" t="n">
         <v>0.0319</v>
       </c>
-      <c r="E14" t="n">
+      <c r="F14" t="n">
         <v>0.008800000000000001</v>
       </c>
-      <c r="F14" t="n">
+      <c r="G14" t="n">
         <v>3.621</v>
       </c>
-      <c r="G14" t="n">
+      <c r="H14" t="n">
         <v>0.0002934666453694434</v>
       </c>
     </row>
@@ -2957,15 +3251,18 @@
         <v>0.0083</v>
       </c>
       <c r="D15" t="n">
+        <v>0.6695</v>
+      </c>
+      <c r="E15" t="n">
         <v>0.0059</v>
       </c>
-      <c r="E15" t="n">
+      <c r="F15" t="n">
         <v>0.0073</v>
       </c>
-      <c r="F15" t="n">
+      <c r="G15" t="n">
         <v>0.8081</v>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
         <v>0.4190591852696735</v>
       </c>
     </row>
@@ -2982,15 +3279,18 @@
         <v>0.008699999999999999</v>
       </c>
       <c r="D16" t="n">
+        <v>3.2828</v>
+      </c>
+      <c r="E16" t="n">
         <v>0.029</v>
       </c>
-      <c r="E16" t="n">
+      <c r="F16" t="n">
         <v>0.0078</v>
       </c>
-      <c r="F16" t="n">
+      <c r="G16" t="n">
         <v>3.7023</v>
       </c>
-      <c r="G16" t="n">
+      <c r="H16" t="n">
         <v>0.000213681386164429</v>
       </c>
     </row>
@@ -3007,15 +3307,18 @@
         <v>0.0172</v>
       </c>
       <c r="D17" t="n">
+        <v>8.032299999999999</v>
+      </c>
+      <c r="E17" t="n">
         <v>0.0523</v>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>0.0117</v>
       </c>
-      <c r="F17" t="n">
+      <c r="G17" t="n">
         <v>4.4864</v>
       </c>
-      <c r="G17" t="n">
+      <c r="H17" t="n">
         <v>7.244521904004026e-06</v>
       </c>
     </row>
@@ -3032,15 +3335,18 @@
         <v>0.0227</v>
       </c>
       <c r="D18" t="n">
+        <v>4.2313</v>
+      </c>
+      <c r="E18" t="n">
         <v>0.0175</v>
       </c>
-      <c r="E18" t="n">
+      <c r="F18" t="n">
         <v>0.009599999999999999</v>
       </c>
-      <c r="F18" t="n">
+      <c r="G18" t="n">
         <v>1.8233</v>
       </c>
-      <c r="G18" t="n">
+      <c r="H18" t="n">
         <v>0.06825282942830668</v>
       </c>
     </row>
@@ -3057,15 +3363,18 @@
         <v>0.0236</v>
       </c>
       <c r="D19" t="n">
+        <v>3.1346</v>
+      </c>
+      <c r="E19" t="n">
         <v>0.0092</v>
       </c>
-      <c r="E19" t="n">
+      <c r="F19" t="n">
         <v>0.0071</v>
       </c>
-      <c r="F19" t="n">
+      <c r="G19" t="n">
         <v>1.307</v>
       </c>
-      <c r="G19" t="n">
+      <c r="H19" t="n">
         <v>0.1912086943180784</v>
       </c>
     </row>
@@ -3082,15 +3391,18 @@
         <v>0.0049</v>
       </c>
       <c r="D20" t="n">
+        <v>-9.111800000000001</v>
+      </c>
+      <c r="E20" t="n">
         <v>-0.1867</v>
       </c>
-      <c r="E20" t="n">
+      <c r="F20" t="n">
         <v>0.009599999999999999</v>
       </c>
-      <c r="F20" t="n">
+      <c r="G20" t="n">
         <v>-19.4143</v>
       </c>
-      <c r="G20" t="n">
+      <c r="H20" t="n">
         <v>5.839484225313443e-84</v>
       </c>
     </row>
@@ -3107,15 +3419,18 @@
         <v>0.0054</v>
       </c>
       <c r="D21" t="n">
+        <v>-9.2684</v>
+      </c>
+      <c r="E21" t="n">
         <v>-0.166</v>
       </c>
-      <c r="E21" t="n">
+      <c r="F21" t="n">
         <v>0.0092</v>
       </c>
-      <c r="F21" t="n">
+      <c r="G21" t="n">
         <v>-18.0107</v>
       </c>
-      <c r="G21" t="n">
+      <c r="H21" t="n">
         <v>1.605448232048225e-72</v>
       </c>
     </row>
@@ -3132,15 +3447,18 @@
         <v>0.0072</v>
       </c>
       <c r="D22" t="n">
+        <v>-11.1107</v>
+      </c>
+      <c r="E22" t="n">
         <v>-0.1548</v>
       </c>
-      <c r="E22" t="n">
+      <c r="F22" t="n">
         <v>0.0095</v>
       </c>
-      <c r="F22" t="n">
+      <c r="G22" t="n">
         <v>-16.3596</v>
       </c>
-      <c r="G22" t="n">
+      <c r="H22" t="n">
         <v>3.714453782580163e-60</v>
       </c>
     </row>
@@ -3157,15 +3475,18 @@
         <v>0.0059</v>
       </c>
       <c r="D23" t="n">
+        <v>-6.8662</v>
+      </c>
+      <c r="E23" t="n">
         <v>-0.1389</v>
       </c>
-      <c r="E23" t="n">
+      <c r="F23" t="n">
         <v>0.0116</v>
       </c>
-      <c r="F23" t="n">
+      <c r="G23" t="n">
         <v>-11.9933</v>
       </c>
-      <c r="G23" t="n">
+      <c r="H23" t="n">
         <v>3.851077963661381e-33</v>
       </c>
     </row>
@@ -3182,15 +3503,18 @@
         <v>0.0076</v>
       </c>
       <c r="D24" t="n">
+        <v>-9.662000000000001</v>
+      </c>
+      <c r="E24" t="n">
         <v>-0.1154</v>
       </c>
-      <c r="E24" t="n">
+      <c r="F24" t="n">
         <v>0.0086</v>
       </c>
-      <c r="F24" t="n">
+      <c r="G24" t="n">
         <v>-13.3482</v>
       </c>
-      <c r="G24" t="n">
+      <c r="H24" t="n">
         <v>1.214058286056416e-40</v>
       </c>
     </row>
@@ -3207,15 +3531,18 @@
         <v>0.0037</v>
       </c>
       <c r="D25" t="n">
+        <v>-4.5001</v>
+      </c>
+      <c r="E25" t="n">
         <v>-0.0864</v>
       </c>
-      <c r="E25" t="n">
+      <c r="F25" t="n">
         <v>0.0069</v>
       </c>
-      <c r="F25" t="n">
+      <c r="G25" t="n">
         <v>-12.4908</v>
       </c>
-      <c r="G25" t="n">
+      <c r="H25" t="n">
         <v>8.380030162345431e-36</v>
       </c>
     </row>
@@ -3232,15 +3559,18 @@
         <v>0.0046</v>
       </c>
       <c r="D26" t="n">
+        <v>-3.0169</v>
+      </c>
+      <c r="E26" t="n">
         <v>-0.0453</v>
       </c>
-      <c r="E26" t="n">
+      <c r="F26" t="n">
         <v>0.0068</v>
       </c>
-      <c r="F26" t="n">
+      <c r="G26" t="n">
         <v>-6.6292</v>
       </c>
-      <c r="G26" t="n">
+      <c r="H26" t="n">
         <v>3.374381682041112e-11</v>
       </c>
     </row>
@@ -3257,15 +3587,18 @@
         <v>0.0038</v>
       </c>
       <c r="D27" t="n">
+        <v>-5.6934</v>
+      </c>
+      <c r="E27" t="n">
         <v>-0.08699999999999999</v>
       </c>
-      <c r="E27" t="n">
+      <c r="F27" t="n">
         <v>0.0057</v>
       </c>
-      <c r="F27" t="n">
+      <c r="G27" t="n">
         <v>-15.2322</v>
       </c>
-      <c r="G27" t="n">
+      <c r="H27" t="n">
         <v>2.162640598758015e-52</v>
       </c>
     </row>
@@ -3280,7 +3613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3301,20 +3634,25 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>pct_effect (%)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>SE_Beta</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>t</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>p</t>
         </is>
@@ -3334,10 +3672,11 @@
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
-      <c r="F2" t="n">
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
         <v>29.6153</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>9.493174009798496e-193</v>
       </c>
     </row>
@@ -3354,15 +3693,18 @@
         <v>0.0016</v>
       </c>
       <c r="D3" t="n">
+        <v>2.5348</v>
+      </c>
+      <c r="E3" t="n">
         <v>0.2048</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>0.0132</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>15.4752</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>5.098290085572425e-54</v>
       </c>
     </row>
@@ -3379,15 +3721,18 @@
         <v>0.0024</v>
       </c>
       <c r="D4" t="n">
+        <v>-4.8923</v>
+      </c>
+      <c r="E4" t="n">
         <v>-0.2425</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>0.0117</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>-20.798</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>4.516185900993735e-96</v>
       </c>
     </row>
@@ -3404,15 +3749,18 @@
         <v>0.0002</v>
       </c>
       <c r="D5" t="n">
+        <v>0.1724</v>
+      </c>
+      <c r="E5" t="n">
         <v>0.08749999999999999</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>0.008699999999999999</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>10.1001</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>5.520102026723362e-24</v>
       </c>
     </row>
@@ -3429,15 +3777,18 @@
         <v>0.0033</v>
       </c>
       <c r="D6" t="n">
+        <v>2.4626</v>
+      </c>
+      <c r="E6" t="n">
         <v>0.09569999999999999</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>0.0128</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>7.4661</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>8.263638734334532e-14</v>
       </c>
     </row>
@@ -3454,15 +3805,18 @@
         <v>0.0034</v>
       </c>
       <c r="D7" t="n">
+        <v>2.8962</v>
+      </c>
+      <c r="E7" t="n">
         <v>0.1095</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>0.0132</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>8.3161</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>9.090366403607607e-17</v>
       </c>
     </row>
@@ -3479,15 +3833,18 @@
         <v>0.0033</v>
       </c>
       <c r="D8" t="n">
+        <v>3.181</v>
+      </c>
+      <c r="E8" t="n">
         <v>0.1006</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>0.0106</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>9.5143</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>1.828701716444621e-21</v>
       </c>
     </row>
@@ -3504,15 +3861,18 @@
         <v>0.003</v>
       </c>
       <c r="D9" t="n">
+        <v>2.122</v>
+      </c>
+      <c r="E9" t="n">
         <v>0.0576</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>0.008200000000000001</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>6.9861</v>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>2.826954633779415e-12</v>
       </c>
     </row>
@@ -3529,15 +3889,18 @@
         <v>0.0046</v>
       </c>
       <c r="D10" t="n">
+        <v>4.5897</v>
+      </c>
+      <c r="E10" t="n">
         <v>0.138</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>0.0142</v>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>9.6936</v>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>3.210556741344724e-22</v>
       </c>
     </row>
@@ -3554,15 +3917,18 @@
         <v>0.0033</v>
       </c>
       <c r="D11" t="n">
+        <v>2.2227</v>
+      </c>
+      <c r="E11" t="n">
         <v>0.06759999999999999</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>0.01</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>6.7563</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>1.415727937803293e-11</v>
       </c>
     </row>
@@ -3579,15 +3945,18 @@
         <v>0.0032</v>
       </c>
       <c r="D12" t="n">
+        <v>2.5739</v>
+      </c>
+      <c r="E12" t="n">
         <v>0.0645</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>0.0081</v>
       </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>7.9973</v>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>1.271356955724793e-15</v>
       </c>
     </row>
@@ -3604,15 +3973,18 @@
         <v>0.0034</v>
       </c>
       <c r="D13" t="n">
+        <v>1.874</v>
+      </c>
+      <c r="E13" t="n">
         <v>0.0471</v>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>0.008699999999999999</v>
       </c>
-      <c r="F13" t="n">
+      <c r="G13" t="n">
         <v>5.3959</v>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>6.818386801856259e-08</v>
       </c>
     </row>
@@ -3629,15 +4001,18 @@
         <v>0.0038</v>
       </c>
       <c r="D14" t="n">
+        <v>1.7565</v>
+      </c>
+      <c r="E14" t="n">
         <v>0.0368</v>
       </c>
-      <c r="E14" t="n">
+      <c r="F14" t="n">
         <v>0.008</v>
       </c>
-      <c r="F14" t="n">
+      <c r="G14" t="n">
         <v>4.6235</v>
       </c>
-      <c r="G14" t="n">
+      <c r="H14" t="n">
         <v>3.774055178535852e-06</v>
       </c>
     </row>
@@ -3654,15 +4029,18 @@
         <v>0.003</v>
       </c>
       <c r="D15" t="n">
+        <v>0.3743</v>
+      </c>
+      <c r="E15" t="n">
         <v>0.0073</v>
       </c>
-      <c r="E15" t="n">
+      <c r="F15" t="n">
         <v>0.0059</v>
       </c>
-      <c r="F15" t="n">
+      <c r="G15" t="n">
         <v>1.2452</v>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
         <v>0.2130499859921222</v>
       </c>
     </row>
@@ -3679,15 +4057,18 @@
         <v>0.0029</v>
       </c>
       <c r="D16" t="n">
+        <v>1.7983</v>
+      </c>
+      <c r="E16" t="n">
         <v>0.0368</v>
       </c>
-      <c r="E16" t="n">
+      <c r="F16" t="n">
         <v>0.0061</v>
       </c>
-      <c r="F16" t="n">
+      <c r="G16" t="n">
         <v>6.0578</v>
       </c>
-      <c r="G16" t="n">
+      <c r="H16" t="n">
         <v>1.379790101527942e-09</v>
       </c>
     </row>
@@ -3704,15 +4085,18 @@
         <v>0.0075</v>
       </c>
       <c r="D17" t="n">
+        <v>2.5642</v>
+      </c>
+      <c r="E17" t="n">
         <v>0.0368</v>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>0.0108</v>
       </c>
-      <c r="F17" t="n">
+      <c r="G17" t="n">
         <v>3.3951</v>
       </c>
-      <c r="G17" t="n">
+      <c r="H17" t="n">
         <v>0.0006860189959474789</v>
       </c>
     </row>
@@ -3729,15 +4113,18 @@
         <v>0.0069</v>
       </c>
       <c r="D18" t="n">
+        <v>1.1011</v>
+      </c>
+      <c r="E18" t="n">
         <v>0.0105</v>
       </c>
-      <c r="E18" t="n">
+      <c r="F18" t="n">
         <v>0.0067</v>
       </c>
-      <c r="F18" t="n">
+      <c r="G18" t="n">
         <v>1.5783</v>
       </c>
-      <c r="G18" t="n">
+      <c r="H18" t="n">
         <v>0.1145049998589514</v>
       </c>
     </row>
@@ -3754,15 +4141,18 @@
         <v>0.0074</v>
       </c>
       <c r="D19" t="n">
+        <v>0.1464</v>
+      </c>
+      <c r="E19" t="n">
         <v>0.001</v>
       </c>
-      <c r="E19" t="n">
+      <c r="F19" t="n">
         <v>0.0051</v>
       </c>
-      <c r="F19" t="n">
+      <c r="G19" t="n">
         <v>0.1989</v>
       </c>
-      <c r="G19" t="n">
+      <c r="H19" t="n">
         <v>0.8423610967934463</v>
       </c>
     </row>
@@ -3779,15 +4169,18 @@
         <v>0.0021</v>
       </c>
       <c r="D20" t="n">
+        <v>-5.5219</v>
+      </c>
+      <c r="E20" t="n">
         <v>-0.2539</v>
       </c>
-      <c r="E20" t="n">
+      <c r="F20" t="n">
         <v>0.009299999999999999</v>
       </c>
-      <c r="F20" t="n">
+      <c r="G20" t="n">
         <v>-27.4281</v>
       </c>
-      <c r="G20" t="n">
+      <c r="H20" t="n">
         <v>1.267181109150088e-165</v>
       </c>
     </row>
@@ -3804,15 +4197,18 @@
         <v>0.0023</v>
       </c>
       <c r="D21" t="n">
+        <v>-5.4738</v>
+      </c>
+      <c r="E21" t="n">
         <v>-0.2144</v>
       </c>
-      <c r="E21" t="n">
+      <c r="F21" t="n">
         <v>0.008699999999999999</v>
       </c>
-      <c r="F21" t="n">
+      <c r="G21" t="n">
         <v>-24.5696</v>
       </c>
-      <c r="G21" t="n">
+      <c r="H21" t="n">
         <v>2.670911495138096e-133</v>
       </c>
     </row>
@@ -3829,15 +4225,18 @@
         <v>0.0027</v>
       </c>
       <c r="D22" t="n">
+        <v>-6.8945</v>
+      </c>
+      <c r="E22" t="n">
         <v>-0.195</v>
       </c>
-      <c r="E22" t="n">
+      <c r="F22" t="n">
         <v>0.0074</v>
       </c>
-      <c r="F22" t="n">
+      <c r="G22" t="n">
         <v>-26.2031</v>
       </c>
-      <c r="G22" t="n">
+      <c r="H22" t="n">
         <v>2.452221048853129e-151</v>
       </c>
     </row>
@@ -3854,15 +4253,18 @@
         <v>0.0026</v>
       </c>
       <c r="D23" t="n">
+        <v>-4.7373</v>
+      </c>
+      <c r="E23" t="n">
         <v>-0.2064</v>
       </c>
-      <c r="E23" t="n">
+      <c r="F23" t="n">
         <v>0.0111</v>
       </c>
-      <c r="F23" t="n">
+      <c r="G23" t="n">
         <v>-18.5539</v>
       </c>
-      <c r="G23" t="n">
+      <c r="H23" t="n">
         <v>7.578256781602136e-77</v>
       </c>
     </row>
@@ -3879,15 +4281,18 @@
         <v>0.0037</v>
       </c>
       <c r="D24" t="n">
+        <v>-3.4916</v>
+      </c>
+      <c r="E24" t="n">
         <v>-0.0917</v>
       </c>
-      <c r="E24" t="n">
+      <c r="F24" t="n">
         <v>0.009599999999999999</v>
       </c>
-      <c r="F24" t="n">
+      <c r="G24" t="n">
         <v>-9.533200000000001</v>
       </c>
-      <c r="G24" t="n">
+      <c r="H24" t="n">
         <v>1.525523201478916e-21</v>
       </c>
     </row>
@@ -3904,15 +4309,18 @@
         <v>0.0014</v>
       </c>
       <c r="D25" t="n">
+        <v>-1.8142</v>
+      </c>
+      <c r="E25" t="n">
         <v>-0.0769</v>
       </c>
-      <c r="E25" t="n">
+      <c r="F25" t="n">
         <v>0.0061</v>
       </c>
-      <c r="F25" t="n">
+      <c r="G25" t="n">
         <v>-12.6984</v>
       </c>
-      <c r="G25" t="n">
+      <c r="H25" t="n">
         <v>6.031610362271175e-37</v>
       </c>
     </row>
@@ -3929,15 +4337,18 @@
         <v>0.0018</v>
       </c>
       <c r="D26" t="n">
+        <v>-1.7152</v>
+      </c>
+      <c r="E26" t="n">
         <v>-0.0573</v>
       </c>
-      <c r="E26" t="n">
+      <c r="F26" t="n">
         <v>0.0058</v>
       </c>
-      <c r="F26" t="n">
+      <c r="G26" t="n">
         <v>-9.868</v>
       </c>
-      <c r="G26" t="n">
+      <c r="H26" t="n">
         <v>5.728423285631834e-23</v>
       </c>
     </row>
@@ -3954,15 +4365,18 @@
         <v>0.0015</v>
       </c>
       <c r="D27" t="n">
+        <v>-2.4219</v>
+      </c>
+      <c r="E27" t="n">
         <v>-0.0863</v>
       </c>
-      <c r="E27" t="n">
+      <c r="F27" t="n">
         <v>0.0054</v>
       </c>
-      <c r="F27" t="n">
+      <c r="G27" t="n">
         <v>-15.8974</v>
       </c>
-      <c r="G27" t="n">
+      <c r="H27" t="n">
         <v>6.609746737921694e-57</v>
       </c>
     </row>

</xml_diff>